<commit_message>
Add Schedule III PPE Note (gross/net block movement schedule)
- New 'Schedule III PPE Note' sheet: disclosure-format movement schedule
  with Gross Block (opening/additions/disposals/closing), Depreciation
  (opening/charge/on-disposals/closing) and Net Block (CY vs PY) by class
  of asset, driven from the FAR for the selected reporting year
- Per-asset working with opening-block, additions, disposals, opening
  accumulated depreciation, charge and elimination on disposal
- Built-in checks: Net = Gross - Depreciation, and charge ties to FAR
- README updated

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E8SeZjPw1ZhN9qJSt7HMTw
</commit_message>
<xml_diff>
--- a/FAR_Schedule_II.xlsx
+++ b/FAR_Schedule_II.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Income-Tax Dep Chart" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Notes &amp; Compliance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Book vs Tax (Def. Tax)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Schedule III PPE Note" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="GlobalCompany">Input!$C$6</definedName>
@@ -43,7 +44,7 @@
     <numFmt numFmtId="168" formatCode="&quot;FY &quot;yyyy"/>
     <numFmt numFmtId="169" formatCode="&quot;Dep &quot;yyyy"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="44">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -281,8 +282,26 @@
       <color rgb="00000000"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00548235"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="7"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -357,6 +376,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E5DEF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
       </patternFill>
     </fill>
   </fills>
@@ -444,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -971,6 +995,70 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="41" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="41" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="43" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="43" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="43" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="43" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -31325,4 +31413,4605 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:O97"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="178" t="inlineStr">
+        <is>
+          <t>NOTE 2.1 – PROPERTY, PLANT AND EQUIPMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="95">
+        <f>"Reconciliation of gross &amp; net carrying amounts (Schedule III, Companies Act 2013)   |   Current year ended "&amp;TEXT(ReportingFYEnd,"dd-mmm-yyyy")&amp;"   |   Previous year ended "&amp;TEXT(EDATE(ReportingFYEnd,-12),"dd-mmm-yyyy")&amp;"   |   (Amounts in Rs.)"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="179" t="inlineStr"/>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>GROSS BLOCK (at cost)</t>
+        </is>
+      </c>
+      <c r="G5" s="36" t="inlineStr">
+        <is>
+          <t>DEPRECIATION / AMORTISATION</t>
+        </is>
+      </c>
+      <c r="K5" s="37" t="inlineStr">
+        <is>
+          <t>NET BLOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="B6" s="108" t="inlineStr">
+        <is>
+          <t>Class of Asset</t>
+        </is>
+      </c>
+      <c r="C6" s="108" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="D6" s="108" t="inlineStr">
+        <is>
+          <t>Additions</t>
+        </is>
+      </c>
+      <c r="E6" s="108" t="inlineStr">
+        <is>
+          <t>Disposals</t>
+        </is>
+      </c>
+      <c r="F6" s="108" t="inlineStr">
+        <is>
+          <t>Closing</t>
+        </is>
+      </c>
+      <c r="G6" s="108" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="H6" s="108" t="inlineStr">
+        <is>
+          <t>For the Year</t>
+        </is>
+      </c>
+      <c r="I6" s="108" t="inlineStr">
+        <is>
+          <t>On Disposals</t>
+        </is>
+      </c>
+      <c r="J6" s="108" t="inlineStr">
+        <is>
+          <t>Closing</t>
+        </is>
+      </c>
+      <c r="K6" s="108" t="inlineStr">
+        <is>
+          <t>As at CY</t>
+        </is>
+      </c>
+      <c r="L6" s="108" t="inlineStr">
+        <is>
+          <t>As at PY</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="92">
+        <f>Input!C15</f>
+        <v/>
+      </c>
+      <c r="C7" s="63">
+        <f>SUMIF($C$38:$C$97,$B7,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D7" s="63">
+        <f>SUMIF($C$38:$C$97,$B7,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E7" s="131">
+        <f>SUMIF($C$38:$C$97,$B7,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F7" s="131">
+        <f>C7+D7-E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="63">
+        <f>SUMIF($C$38:$C$97,$B7,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H7" s="63">
+        <f>SUMIF($C$38:$C$97,$B7,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I7" s="131">
+        <f>SUMIF($C$38:$C$97,$B7,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J7" s="131">
+        <f>G7+H7-I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="180">
+        <f>F7-J7</f>
+        <v/>
+      </c>
+      <c r="L7" s="181">
+        <f>C7-G7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="93">
+        <f>Input!C16</f>
+        <v/>
+      </c>
+      <c r="C8" s="81">
+        <f>SUMIF($C$38:$C$97,$B8,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D8" s="81">
+        <f>SUMIF($C$38:$C$97,$B8,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E8" s="120">
+        <f>SUMIF($C$38:$C$97,$B8,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F8" s="120">
+        <f>C8+D8-E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="81">
+        <f>SUMIF($C$38:$C$97,$B8,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H8" s="81">
+        <f>SUMIF($C$38:$C$97,$B8,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I8" s="120">
+        <f>SUMIF($C$38:$C$97,$B8,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J8" s="120">
+        <f>G8+H8-I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="182">
+        <f>F8-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="183">
+        <f>C8-G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="92">
+        <f>Input!C17</f>
+        <v/>
+      </c>
+      <c r="C9" s="63">
+        <f>SUMIF($C$38:$C$97,$B9,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D9" s="63">
+        <f>SUMIF($C$38:$C$97,$B9,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E9" s="131">
+        <f>SUMIF($C$38:$C$97,$B9,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F9" s="131">
+        <f>C9+D9-E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="63">
+        <f>SUMIF($C$38:$C$97,$B9,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H9" s="63">
+        <f>SUMIF($C$38:$C$97,$B9,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I9" s="131">
+        <f>SUMIF($C$38:$C$97,$B9,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J9" s="131">
+        <f>G9+H9-I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="180">
+        <f>F9-J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="181">
+        <f>C9-G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="93">
+        <f>Input!C18</f>
+        <v/>
+      </c>
+      <c r="C10" s="81">
+        <f>SUMIF($C$38:$C$97,$B10,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D10" s="81">
+        <f>SUMIF($C$38:$C$97,$B10,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E10" s="120">
+        <f>SUMIF($C$38:$C$97,$B10,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F10" s="120">
+        <f>C10+D10-E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="81">
+        <f>SUMIF($C$38:$C$97,$B10,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H10" s="81">
+        <f>SUMIF($C$38:$C$97,$B10,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I10" s="120">
+        <f>SUMIF($C$38:$C$97,$B10,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J10" s="120">
+        <f>G10+H10-I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="182">
+        <f>F10-J10</f>
+        <v/>
+      </c>
+      <c r="L10" s="183">
+        <f>C10-G10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="92">
+        <f>Input!C19</f>
+        <v/>
+      </c>
+      <c r="C11" s="63">
+        <f>SUMIF($C$38:$C$97,$B11,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D11" s="63">
+        <f>SUMIF($C$38:$C$97,$B11,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E11" s="131">
+        <f>SUMIF($C$38:$C$97,$B11,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F11" s="131">
+        <f>C11+D11-E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="63">
+        <f>SUMIF($C$38:$C$97,$B11,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H11" s="63">
+        <f>SUMIF($C$38:$C$97,$B11,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I11" s="131">
+        <f>SUMIF($C$38:$C$97,$B11,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J11" s="131">
+        <f>G11+H11-I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="180">
+        <f>F11-J11</f>
+        <v/>
+      </c>
+      <c r="L11" s="181">
+        <f>C11-G11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="93">
+        <f>Input!C20</f>
+        <v/>
+      </c>
+      <c r="C12" s="81">
+        <f>SUMIF($C$38:$C$97,$B12,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D12" s="81">
+        <f>SUMIF($C$38:$C$97,$B12,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E12" s="120">
+        <f>SUMIF($C$38:$C$97,$B12,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F12" s="120">
+        <f>C12+D12-E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="81">
+        <f>SUMIF($C$38:$C$97,$B12,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H12" s="81">
+        <f>SUMIF($C$38:$C$97,$B12,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I12" s="120">
+        <f>SUMIF($C$38:$C$97,$B12,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J12" s="120">
+        <f>G12+H12-I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="182">
+        <f>F12-J12</f>
+        <v/>
+      </c>
+      <c r="L12" s="183">
+        <f>C12-G12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="92">
+        <f>Input!C21</f>
+        <v/>
+      </c>
+      <c r="C13" s="63">
+        <f>SUMIF($C$38:$C$97,$B13,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D13" s="63">
+        <f>SUMIF($C$38:$C$97,$B13,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E13" s="131">
+        <f>SUMIF($C$38:$C$97,$B13,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F13" s="131">
+        <f>C13+D13-E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="63">
+        <f>SUMIF($C$38:$C$97,$B13,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H13" s="63">
+        <f>SUMIF($C$38:$C$97,$B13,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I13" s="131">
+        <f>SUMIF($C$38:$C$97,$B13,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J13" s="131">
+        <f>G13+H13-I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="180">
+        <f>F13-J13</f>
+        <v/>
+      </c>
+      <c r="L13" s="181">
+        <f>C13-G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="93">
+        <f>Input!C22</f>
+        <v/>
+      </c>
+      <c r="C14" s="81">
+        <f>SUMIF($C$38:$C$97,$B14,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D14" s="81">
+        <f>SUMIF($C$38:$C$97,$B14,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E14" s="120">
+        <f>SUMIF($C$38:$C$97,$B14,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F14" s="120">
+        <f>C14+D14-E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="81">
+        <f>SUMIF($C$38:$C$97,$B14,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H14" s="81">
+        <f>SUMIF($C$38:$C$97,$B14,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I14" s="120">
+        <f>SUMIF($C$38:$C$97,$B14,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J14" s="120">
+        <f>G14+H14-I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="182">
+        <f>F14-J14</f>
+        <v/>
+      </c>
+      <c r="L14" s="183">
+        <f>C14-G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="92">
+        <f>Input!C23</f>
+        <v/>
+      </c>
+      <c r="C15" s="63">
+        <f>SUMIF($C$38:$C$97,$B15,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D15" s="63">
+        <f>SUMIF($C$38:$C$97,$B15,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E15" s="131">
+        <f>SUMIF($C$38:$C$97,$B15,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F15" s="131">
+        <f>C15+D15-E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="63">
+        <f>SUMIF($C$38:$C$97,$B15,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H15" s="63">
+        <f>SUMIF($C$38:$C$97,$B15,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I15" s="131">
+        <f>SUMIF($C$38:$C$97,$B15,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J15" s="131">
+        <f>G15+H15-I15</f>
+        <v/>
+      </c>
+      <c r="K15" s="180">
+        <f>F15-J15</f>
+        <v/>
+      </c>
+      <c r="L15" s="181">
+        <f>C15-G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="93">
+        <f>Input!C24</f>
+        <v/>
+      </c>
+      <c r="C16" s="81">
+        <f>SUMIF($C$38:$C$97,$B16,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D16" s="81">
+        <f>SUMIF($C$38:$C$97,$B16,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E16" s="120">
+        <f>SUMIF($C$38:$C$97,$B16,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F16" s="120">
+        <f>C16+D16-E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="81">
+        <f>SUMIF($C$38:$C$97,$B16,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H16" s="81">
+        <f>SUMIF($C$38:$C$97,$B16,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I16" s="120">
+        <f>SUMIF($C$38:$C$97,$B16,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J16" s="120">
+        <f>G16+H16-I16</f>
+        <v/>
+      </c>
+      <c r="K16" s="182">
+        <f>F16-J16</f>
+        <v/>
+      </c>
+      <c r="L16" s="183">
+        <f>C16-G16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="92">
+        <f>Input!C25</f>
+        <v/>
+      </c>
+      <c r="C17" s="63">
+        <f>SUMIF($C$38:$C$97,$B17,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D17" s="63">
+        <f>SUMIF($C$38:$C$97,$B17,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E17" s="131">
+        <f>SUMIF($C$38:$C$97,$B17,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F17" s="131">
+        <f>C17+D17-E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="63">
+        <f>SUMIF($C$38:$C$97,$B17,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H17" s="63">
+        <f>SUMIF($C$38:$C$97,$B17,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I17" s="131">
+        <f>SUMIF($C$38:$C$97,$B17,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J17" s="131">
+        <f>G17+H17-I17</f>
+        <v/>
+      </c>
+      <c r="K17" s="180">
+        <f>F17-J17</f>
+        <v/>
+      </c>
+      <c r="L17" s="181">
+        <f>C17-G17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="93">
+        <f>Input!C26</f>
+        <v/>
+      </c>
+      <c r="C18" s="81">
+        <f>SUMIF($C$38:$C$97,$B18,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D18" s="81">
+        <f>SUMIF($C$38:$C$97,$B18,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E18" s="120">
+        <f>SUMIF($C$38:$C$97,$B18,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F18" s="120">
+        <f>C18+D18-E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="81">
+        <f>SUMIF($C$38:$C$97,$B18,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H18" s="81">
+        <f>SUMIF($C$38:$C$97,$B18,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I18" s="120">
+        <f>SUMIF($C$38:$C$97,$B18,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J18" s="120">
+        <f>G18+H18-I18</f>
+        <v/>
+      </c>
+      <c r="K18" s="182">
+        <f>F18-J18</f>
+        <v/>
+      </c>
+      <c r="L18" s="183">
+        <f>C18-G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="92">
+        <f>Input!C27</f>
+        <v/>
+      </c>
+      <c r="C19" s="63">
+        <f>SUMIF($C$38:$C$97,$B19,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D19" s="63">
+        <f>SUMIF($C$38:$C$97,$B19,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E19" s="131">
+        <f>SUMIF($C$38:$C$97,$B19,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F19" s="131">
+        <f>C19+D19-E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="63">
+        <f>SUMIF($C$38:$C$97,$B19,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H19" s="63">
+        <f>SUMIF($C$38:$C$97,$B19,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I19" s="131">
+        <f>SUMIF($C$38:$C$97,$B19,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J19" s="131">
+        <f>G19+H19-I19</f>
+        <v/>
+      </c>
+      <c r="K19" s="180">
+        <f>F19-J19</f>
+        <v/>
+      </c>
+      <c r="L19" s="181">
+        <f>C19-G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="93">
+        <f>Input!C28</f>
+        <v/>
+      </c>
+      <c r="C20" s="81">
+        <f>SUMIF($C$38:$C$97,$B20,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D20" s="81">
+        <f>SUMIF($C$38:$C$97,$B20,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E20" s="120">
+        <f>SUMIF($C$38:$C$97,$B20,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F20" s="120">
+        <f>C20+D20-E20</f>
+        <v/>
+      </c>
+      <c r="G20" s="81">
+        <f>SUMIF($C$38:$C$97,$B20,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H20" s="81">
+        <f>SUMIF($C$38:$C$97,$B20,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I20" s="120">
+        <f>SUMIF($C$38:$C$97,$B20,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J20" s="120">
+        <f>G20+H20-I20</f>
+        <v/>
+      </c>
+      <c r="K20" s="182">
+        <f>F20-J20</f>
+        <v/>
+      </c>
+      <c r="L20" s="183">
+        <f>C20-G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="92">
+        <f>Input!C29</f>
+        <v/>
+      </c>
+      <c r="C21" s="63">
+        <f>SUMIF($C$38:$C$97,$B21,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D21" s="63">
+        <f>SUMIF($C$38:$C$97,$B21,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E21" s="131">
+        <f>SUMIF($C$38:$C$97,$B21,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F21" s="131">
+        <f>C21+D21-E21</f>
+        <v/>
+      </c>
+      <c r="G21" s="63">
+        <f>SUMIF($C$38:$C$97,$B21,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H21" s="63">
+        <f>SUMIF($C$38:$C$97,$B21,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I21" s="131">
+        <f>SUMIF($C$38:$C$97,$B21,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J21" s="131">
+        <f>G21+H21-I21</f>
+        <v/>
+      </c>
+      <c r="K21" s="180">
+        <f>F21-J21</f>
+        <v/>
+      </c>
+      <c r="L21" s="181">
+        <f>C21-G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="93">
+        <f>Input!C30</f>
+        <v/>
+      </c>
+      <c r="C22" s="81">
+        <f>SUMIF($C$38:$C$97,$B22,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D22" s="81">
+        <f>SUMIF($C$38:$C$97,$B22,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E22" s="120">
+        <f>SUMIF($C$38:$C$97,$B22,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F22" s="120">
+        <f>C22+D22-E22</f>
+        <v/>
+      </c>
+      <c r="G22" s="81">
+        <f>SUMIF($C$38:$C$97,$B22,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H22" s="81">
+        <f>SUMIF($C$38:$C$97,$B22,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I22" s="120">
+        <f>SUMIF($C$38:$C$97,$B22,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J22" s="120">
+        <f>G22+H22-I22</f>
+        <v/>
+      </c>
+      <c r="K22" s="182">
+        <f>F22-J22</f>
+        <v/>
+      </c>
+      <c r="L22" s="183">
+        <f>C22-G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="92">
+        <f>Input!C31</f>
+        <v/>
+      </c>
+      <c r="C23" s="63">
+        <f>SUMIF($C$38:$C$97,$B23,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D23" s="63">
+        <f>SUMIF($C$38:$C$97,$B23,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E23" s="131">
+        <f>SUMIF($C$38:$C$97,$B23,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F23" s="131">
+        <f>C23+D23-E23</f>
+        <v/>
+      </c>
+      <c r="G23" s="63">
+        <f>SUMIF($C$38:$C$97,$B23,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H23" s="63">
+        <f>SUMIF($C$38:$C$97,$B23,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I23" s="131">
+        <f>SUMIF($C$38:$C$97,$B23,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J23" s="131">
+        <f>G23+H23-I23</f>
+        <v/>
+      </c>
+      <c r="K23" s="180">
+        <f>F23-J23</f>
+        <v/>
+      </c>
+      <c r="L23" s="181">
+        <f>C23-G23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="93">
+        <f>Input!C32</f>
+        <v/>
+      </c>
+      <c r="C24" s="81">
+        <f>SUMIF($C$38:$C$97,$B24,$I$38:$I$97)</f>
+        <v/>
+      </c>
+      <c r="D24" s="81">
+        <f>SUMIF($C$38:$C$97,$B24,$J$38:$J$97)</f>
+        <v/>
+      </c>
+      <c r="E24" s="120">
+        <f>SUMIF($C$38:$C$97,$B24,$K$38:$K$97)</f>
+        <v/>
+      </c>
+      <c r="F24" s="120">
+        <f>C24+D24-E24</f>
+        <v/>
+      </c>
+      <c r="G24" s="81">
+        <f>SUMIF($C$38:$C$97,$B24,$L$38:$L$97)</f>
+        <v/>
+      </c>
+      <c r="H24" s="81">
+        <f>SUMIF($C$38:$C$97,$B24,$M$38:$M$97)</f>
+        <v/>
+      </c>
+      <c r="I24" s="120">
+        <f>SUMIF($C$38:$C$97,$B24,$O$38:$O$97)</f>
+        <v/>
+      </c>
+      <c r="J24" s="120">
+        <f>G24+H24-I24</f>
+        <v/>
+      </c>
+      <c r="K24" s="182">
+        <f>F24-J24</f>
+        <v/>
+      </c>
+      <c r="L24" s="183">
+        <f>C24-G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C25" s="124">
+        <f>SUM(C7:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="124">
+        <f>SUM(D7:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="124">
+        <f>SUM(E7:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="124">
+        <f>SUM(F7:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="124">
+        <f>SUM(G7:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="124">
+        <f>SUM(H7:H24)</f>
+        <v/>
+      </c>
+      <c r="I25" s="124">
+        <f>SUM(I7:I24)</f>
+        <v/>
+      </c>
+      <c r="J25" s="124">
+        <f>SUM(J7:J24)</f>
+        <v/>
+      </c>
+      <c r="K25" s="124">
+        <f>SUM(K7:K24)</f>
+        <v/>
+      </c>
+      <c r="L25" s="124">
+        <f>SUM(L7:L24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="184" t="inlineStr">
+        <is>
+          <t>Checks:</t>
+        </is>
+      </c>
+      <c r="H26" s="185">
+        <f>IF(ROUND(H25-SUM(FAR!R5:R64),0)=0,"Charge ties to FAR  ✓","CHECK")</f>
+        <v/>
+      </c>
+      <c r="K26" s="185">
+        <f>IF(ROUND(K25-(F25-J25),0)=0,"Net = Gross − Dep  ✓","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="B28" s="177" t="inlineStr">
+        <is>
+          <t>1.  Presentation as per Schedule III to the Companies Act, 2013. Intangible assets (e.g. software) are required to be disclosed in a separate note in the same movement format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="B29" s="177" t="inlineStr">
+        <is>
+          <t>2.  Additions and disposals are captured from the asset 'Date Put to Use' and 'Date of Sale/Disposal' on the FAR for the selected reporting year; depreciation 'For the Year' is the Schedule II charge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="B30" s="177" t="inlineStr">
+        <is>
+          <t>3.  Disclose separately, where applicable: assets held for sale, revalued amounts (Registered Valuer), title deeds of immovable property not in the company's name, and assets given as security (see Notes &amp; Compliance / CARO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="186" t="inlineStr">
+        <is>
+          <t>Working – per-asset movement for the reporting year (auto-linked to FAR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="B37" s="187" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="C37" s="187" t="inlineStr">
+        <is>
+          <t>Class (key)</t>
+        </is>
+      </c>
+      <c r="D37" s="187" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="E37" s="187" t="inlineStr">
+        <is>
+          <t>Put to Use</t>
+        </is>
+      </c>
+      <c r="F37" s="187" t="inlineStr">
+        <is>
+          <t>Disposal</t>
+        </is>
+      </c>
+      <c r="G37" s="187" t="inlineStr">
+        <is>
+          <t>WDV @ PY-end</t>
+        </is>
+      </c>
+      <c r="H37" s="187" t="inlineStr">
+        <is>
+          <t>In Opening?</t>
+        </is>
+      </c>
+      <c r="I37" s="187" t="inlineStr">
+        <is>
+          <t>Gross Opening</t>
+        </is>
+      </c>
+      <c r="J37" s="187" t="inlineStr">
+        <is>
+          <t>Additions</t>
+        </is>
+      </c>
+      <c r="K37" s="187" t="inlineStr">
+        <is>
+          <t>Disposals</t>
+        </is>
+      </c>
+      <c r="L37" s="187" t="inlineStr">
+        <is>
+          <t>AccDep Opening</t>
+        </is>
+      </c>
+      <c r="M37" s="187" t="inlineStr">
+        <is>
+          <t>Charge (FY)</t>
+        </is>
+      </c>
+      <c r="N37" s="187" t="inlineStr">
+        <is>
+          <t>Disp. this yr?</t>
+        </is>
+      </c>
+      <c r="O37" s="187" t="inlineStr">
+        <is>
+          <t>AccDep Eliminated</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="188">
+        <f>IF(FAR!K5="","",FAR!B5)</f>
+        <v/>
+      </c>
+      <c r="C38" s="189">
+        <f>IF(FAR!K5="","",FAR!C5)</f>
+        <v/>
+      </c>
+      <c r="D38" s="171">
+        <f>IF(FAR!K5="","",FAR!K5)</f>
+        <v/>
+      </c>
+      <c r="E38" s="190">
+        <f>IF(FAR!H5="","",FAR!H5)</f>
+        <v/>
+      </c>
+      <c r="F38" s="191">
+        <f>IF(FAR!I5="","",FAR!I5)</f>
+        <v/>
+      </c>
+      <c r="G38" s="192">
+        <f>IF(FAR!K5="","",IFERROR(INDEX(FAR!$AA5:$BF5,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K5))</f>
+        <v/>
+      </c>
+      <c r="H38" s="193">
+        <f>IF(FAR!K5="",0,IF(AND(FAR!H5&lt;&gt;"",FAR!H5&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I5="",FAR!I5&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I38" s="171">
+        <f>IF($H38=1,FAR!K5,0)</f>
+        <v/>
+      </c>
+      <c r="J38" s="171">
+        <f>IF(AND(FAR!H5&lt;&gt;"",FAR!H5&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H5&lt;=ReportingFYEnd),FAR!K5,0)</f>
+        <v/>
+      </c>
+      <c r="K38" s="192">
+        <f>IF(AND(FAR!I5&lt;&gt;"",FAR!I5&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I5&lt;=ReportingFYEnd),FAR!K5,0)</f>
+        <v/>
+      </c>
+      <c r="L38" s="171">
+        <f>IF($H38=1,FAR!K5-$G38,0)</f>
+        <v/>
+      </c>
+      <c r="M38" s="171">
+        <f>IF(FAR!K5="",0,FAR!R5)</f>
+        <v/>
+      </c>
+      <c r="N38" s="193">
+        <f>IF(AND(FAR!I5&lt;&gt;"",FAR!I5&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I5&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O38" s="192">
+        <f>IF($N38=1,$L38+$M38,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="194">
+        <f>IF(FAR!K6="","",FAR!B6)</f>
+        <v/>
+      </c>
+      <c r="C39" s="195">
+        <f>IF(FAR!K6="","",FAR!C6)</f>
+        <v/>
+      </c>
+      <c r="D39" s="175">
+        <f>IF(FAR!K6="","",FAR!K6)</f>
+        <v/>
+      </c>
+      <c r="E39" s="196">
+        <f>IF(FAR!H6="","",FAR!H6)</f>
+        <v/>
+      </c>
+      <c r="F39" s="197">
+        <f>IF(FAR!I6="","",FAR!I6)</f>
+        <v/>
+      </c>
+      <c r="G39" s="198">
+        <f>IF(FAR!K6="","",IFERROR(INDEX(FAR!$AA6:$BF6,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K6))</f>
+        <v/>
+      </c>
+      <c r="H39" s="199">
+        <f>IF(FAR!K6="",0,IF(AND(FAR!H6&lt;&gt;"",FAR!H6&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I6="",FAR!I6&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I39" s="175">
+        <f>IF($H39=1,FAR!K6,0)</f>
+        <v/>
+      </c>
+      <c r="J39" s="175">
+        <f>IF(AND(FAR!H6&lt;&gt;"",FAR!H6&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H6&lt;=ReportingFYEnd),FAR!K6,0)</f>
+        <v/>
+      </c>
+      <c r="K39" s="198">
+        <f>IF(AND(FAR!I6&lt;&gt;"",FAR!I6&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I6&lt;=ReportingFYEnd),FAR!K6,0)</f>
+        <v/>
+      </c>
+      <c r="L39" s="175">
+        <f>IF($H39=1,FAR!K6-$G39,0)</f>
+        <v/>
+      </c>
+      <c r="M39" s="175">
+        <f>IF(FAR!K6="",0,FAR!R6)</f>
+        <v/>
+      </c>
+      <c r="N39" s="199">
+        <f>IF(AND(FAR!I6&lt;&gt;"",FAR!I6&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I6&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O39" s="198">
+        <f>IF($N39=1,$L39+$M39,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="188">
+        <f>IF(FAR!K7="","",FAR!B7)</f>
+        <v/>
+      </c>
+      <c r="C40" s="189">
+        <f>IF(FAR!K7="","",FAR!C7)</f>
+        <v/>
+      </c>
+      <c r="D40" s="171">
+        <f>IF(FAR!K7="","",FAR!K7)</f>
+        <v/>
+      </c>
+      <c r="E40" s="190">
+        <f>IF(FAR!H7="","",FAR!H7)</f>
+        <v/>
+      </c>
+      <c r="F40" s="191">
+        <f>IF(FAR!I7="","",FAR!I7)</f>
+        <v/>
+      </c>
+      <c r="G40" s="192">
+        <f>IF(FAR!K7="","",IFERROR(INDEX(FAR!$AA7:$BF7,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K7))</f>
+        <v/>
+      </c>
+      <c r="H40" s="193">
+        <f>IF(FAR!K7="",0,IF(AND(FAR!H7&lt;&gt;"",FAR!H7&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I7="",FAR!I7&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I40" s="171">
+        <f>IF($H40=1,FAR!K7,0)</f>
+        <v/>
+      </c>
+      <c r="J40" s="171">
+        <f>IF(AND(FAR!H7&lt;&gt;"",FAR!H7&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H7&lt;=ReportingFYEnd),FAR!K7,0)</f>
+        <v/>
+      </c>
+      <c r="K40" s="192">
+        <f>IF(AND(FAR!I7&lt;&gt;"",FAR!I7&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I7&lt;=ReportingFYEnd),FAR!K7,0)</f>
+        <v/>
+      </c>
+      <c r="L40" s="171">
+        <f>IF($H40=1,FAR!K7-$G40,0)</f>
+        <v/>
+      </c>
+      <c r="M40" s="171">
+        <f>IF(FAR!K7="",0,FAR!R7)</f>
+        <v/>
+      </c>
+      <c r="N40" s="193">
+        <f>IF(AND(FAR!I7&lt;&gt;"",FAR!I7&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I7&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O40" s="192">
+        <f>IF($N40=1,$L40+$M40,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="194">
+        <f>IF(FAR!K8="","",FAR!B8)</f>
+        <v/>
+      </c>
+      <c r="C41" s="195">
+        <f>IF(FAR!K8="","",FAR!C8)</f>
+        <v/>
+      </c>
+      <c r="D41" s="175">
+        <f>IF(FAR!K8="","",FAR!K8)</f>
+        <v/>
+      </c>
+      <c r="E41" s="196">
+        <f>IF(FAR!H8="","",FAR!H8)</f>
+        <v/>
+      </c>
+      <c r="F41" s="197">
+        <f>IF(FAR!I8="","",FAR!I8)</f>
+        <v/>
+      </c>
+      <c r="G41" s="198">
+        <f>IF(FAR!K8="","",IFERROR(INDEX(FAR!$AA8:$BF8,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K8))</f>
+        <v/>
+      </c>
+      <c r="H41" s="199">
+        <f>IF(FAR!K8="",0,IF(AND(FAR!H8&lt;&gt;"",FAR!H8&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I8="",FAR!I8&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I41" s="175">
+        <f>IF($H41=1,FAR!K8,0)</f>
+        <v/>
+      </c>
+      <c r="J41" s="175">
+        <f>IF(AND(FAR!H8&lt;&gt;"",FAR!H8&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H8&lt;=ReportingFYEnd),FAR!K8,0)</f>
+        <v/>
+      </c>
+      <c r="K41" s="198">
+        <f>IF(AND(FAR!I8&lt;&gt;"",FAR!I8&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I8&lt;=ReportingFYEnd),FAR!K8,0)</f>
+        <v/>
+      </c>
+      <c r="L41" s="175">
+        <f>IF($H41=1,FAR!K8-$G41,0)</f>
+        <v/>
+      </c>
+      <c r="M41" s="175">
+        <f>IF(FAR!K8="",0,FAR!R8)</f>
+        <v/>
+      </c>
+      <c r="N41" s="199">
+        <f>IF(AND(FAR!I8&lt;&gt;"",FAR!I8&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I8&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O41" s="198">
+        <f>IF($N41=1,$L41+$M41,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="188">
+        <f>IF(FAR!K9="","",FAR!B9)</f>
+        <v/>
+      </c>
+      <c r="C42" s="189">
+        <f>IF(FAR!K9="","",FAR!C9)</f>
+        <v/>
+      </c>
+      <c r="D42" s="171">
+        <f>IF(FAR!K9="","",FAR!K9)</f>
+        <v/>
+      </c>
+      <c r="E42" s="190">
+        <f>IF(FAR!H9="","",FAR!H9)</f>
+        <v/>
+      </c>
+      <c r="F42" s="191">
+        <f>IF(FAR!I9="","",FAR!I9)</f>
+        <v/>
+      </c>
+      <c r="G42" s="192">
+        <f>IF(FAR!K9="","",IFERROR(INDEX(FAR!$AA9:$BF9,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K9))</f>
+        <v/>
+      </c>
+      <c r="H42" s="193">
+        <f>IF(FAR!K9="",0,IF(AND(FAR!H9&lt;&gt;"",FAR!H9&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I9="",FAR!I9&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I42" s="171">
+        <f>IF($H42=1,FAR!K9,0)</f>
+        <v/>
+      </c>
+      <c r="J42" s="171">
+        <f>IF(AND(FAR!H9&lt;&gt;"",FAR!H9&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H9&lt;=ReportingFYEnd),FAR!K9,0)</f>
+        <v/>
+      </c>
+      <c r="K42" s="192">
+        <f>IF(AND(FAR!I9&lt;&gt;"",FAR!I9&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I9&lt;=ReportingFYEnd),FAR!K9,0)</f>
+        <v/>
+      </c>
+      <c r="L42" s="171">
+        <f>IF($H42=1,FAR!K9-$G42,0)</f>
+        <v/>
+      </c>
+      <c r="M42" s="171">
+        <f>IF(FAR!K9="",0,FAR!R9)</f>
+        <v/>
+      </c>
+      <c r="N42" s="193">
+        <f>IF(AND(FAR!I9&lt;&gt;"",FAR!I9&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I9&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O42" s="192">
+        <f>IF($N42=1,$L42+$M42,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="194">
+        <f>IF(FAR!K10="","",FAR!B10)</f>
+        <v/>
+      </c>
+      <c r="C43" s="195">
+        <f>IF(FAR!K10="","",FAR!C10)</f>
+        <v/>
+      </c>
+      <c r="D43" s="175">
+        <f>IF(FAR!K10="","",FAR!K10)</f>
+        <v/>
+      </c>
+      <c r="E43" s="196">
+        <f>IF(FAR!H10="","",FAR!H10)</f>
+        <v/>
+      </c>
+      <c r="F43" s="197">
+        <f>IF(FAR!I10="","",FAR!I10)</f>
+        <v/>
+      </c>
+      <c r="G43" s="198">
+        <f>IF(FAR!K10="","",IFERROR(INDEX(FAR!$AA10:$BF10,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K10))</f>
+        <v/>
+      </c>
+      <c r="H43" s="199">
+        <f>IF(FAR!K10="",0,IF(AND(FAR!H10&lt;&gt;"",FAR!H10&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I10="",FAR!I10&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I43" s="175">
+        <f>IF($H43=1,FAR!K10,0)</f>
+        <v/>
+      </c>
+      <c r="J43" s="175">
+        <f>IF(AND(FAR!H10&lt;&gt;"",FAR!H10&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H10&lt;=ReportingFYEnd),FAR!K10,0)</f>
+        <v/>
+      </c>
+      <c r="K43" s="198">
+        <f>IF(AND(FAR!I10&lt;&gt;"",FAR!I10&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I10&lt;=ReportingFYEnd),FAR!K10,0)</f>
+        <v/>
+      </c>
+      <c r="L43" s="175">
+        <f>IF($H43=1,FAR!K10-$G43,0)</f>
+        <v/>
+      </c>
+      <c r="M43" s="175">
+        <f>IF(FAR!K10="",0,FAR!R10)</f>
+        <v/>
+      </c>
+      <c r="N43" s="199">
+        <f>IF(AND(FAR!I10&lt;&gt;"",FAR!I10&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I10&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O43" s="198">
+        <f>IF($N43=1,$L43+$M43,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="188">
+        <f>IF(FAR!K11="","",FAR!B11)</f>
+        <v/>
+      </c>
+      <c r="C44" s="189">
+        <f>IF(FAR!K11="","",FAR!C11)</f>
+        <v/>
+      </c>
+      <c r="D44" s="171">
+        <f>IF(FAR!K11="","",FAR!K11)</f>
+        <v/>
+      </c>
+      <c r="E44" s="190">
+        <f>IF(FAR!H11="","",FAR!H11)</f>
+        <v/>
+      </c>
+      <c r="F44" s="191">
+        <f>IF(FAR!I11="","",FAR!I11)</f>
+        <v/>
+      </c>
+      <c r="G44" s="192">
+        <f>IF(FAR!K11="","",IFERROR(INDEX(FAR!$AA11:$BF11,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K11))</f>
+        <v/>
+      </c>
+      <c r="H44" s="193">
+        <f>IF(FAR!K11="",0,IF(AND(FAR!H11&lt;&gt;"",FAR!H11&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I11="",FAR!I11&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I44" s="171">
+        <f>IF($H44=1,FAR!K11,0)</f>
+        <v/>
+      </c>
+      <c r="J44" s="171">
+        <f>IF(AND(FAR!H11&lt;&gt;"",FAR!H11&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H11&lt;=ReportingFYEnd),FAR!K11,0)</f>
+        <v/>
+      </c>
+      <c r="K44" s="192">
+        <f>IF(AND(FAR!I11&lt;&gt;"",FAR!I11&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I11&lt;=ReportingFYEnd),FAR!K11,0)</f>
+        <v/>
+      </c>
+      <c r="L44" s="171">
+        <f>IF($H44=1,FAR!K11-$G44,0)</f>
+        <v/>
+      </c>
+      <c r="M44" s="171">
+        <f>IF(FAR!K11="",0,FAR!R11)</f>
+        <v/>
+      </c>
+      <c r="N44" s="193">
+        <f>IF(AND(FAR!I11&lt;&gt;"",FAR!I11&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I11&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O44" s="192">
+        <f>IF($N44=1,$L44+$M44,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="194">
+        <f>IF(FAR!K12="","",FAR!B12)</f>
+        <v/>
+      </c>
+      <c r="C45" s="195">
+        <f>IF(FAR!K12="","",FAR!C12)</f>
+        <v/>
+      </c>
+      <c r="D45" s="175">
+        <f>IF(FAR!K12="","",FAR!K12)</f>
+        <v/>
+      </c>
+      <c r="E45" s="196">
+        <f>IF(FAR!H12="","",FAR!H12)</f>
+        <v/>
+      </c>
+      <c r="F45" s="197">
+        <f>IF(FAR!I12="","",FAR!I12)</f>
+        <v/>
+      </c>
+      <c r="G45" s="198">
+        <f>IF(FAR!K12="","",IFERROR(INDEX(FAR!$AA12:$BF12,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K12))</f>
+        <v/>
+      </c>
+      <c r="H45" s="199">
+        <f>IF(FAR!K12="",0,IF(AND(FAR!H12&lt;&gt;"",FAR!H12&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I12="",FAR!I12&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I45" s="175">
+        <f>IF($H45=1,FAR!K12,0)</f>
+        <v/>
+      </c>
+      <c r="J45" s="175">
+        <f>IF(AND(FAR!H12&lt;&gt;"",FAR!H12&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H12&lt;=ReportingFYEnd),FAR!K12,0)</f>
+        <v/>
+      </c>
+      <c r="K45" s="198">
+        <f>IF(AND(FAR!I12&lt;&gt;"",FAR!I12&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I12&lt;=ReportingFYEnd),FAR!K12,0)</f>
+        <v/>
+      </c>
+      <c r="L45" s="175">
+        <f>IF($H45=1,FAR!K12-$G45,0)</f>
+        <v/>
+      </c>
+      <c r="M45" s="175">
+        <f>IF(FAR!K12="",0,FAR!R12)</f>
+        <v/>
+      </c>
+      <c r="N45" s="199">
+        <f>IF(AND(FAR!I12&lt;&gt;"",FAR!I12&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I12&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O45" s="198">
+        <f>IF($N45=1,$L45+$M45,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="188">
+        <f>IF(FAR!K13="","",FAR!B13)</f>
+        <v/>
+      </c>
+      <c r="C46" s="189">
+        <f>IF(FAR!K13="","",FAR!C13)</f>
+        <v/>
+      </c>
+      <c r="D46" s="171">
+        <f>IF(FAR!K13="","",FAR!K13)</f>
+        <v/>
+      </c>
+      <c r="E46" s="190">
+        <f>IF(FAR!H13="","",FAR!H13)</f>
+        <v/>
+      </c>
+      <c r="F46" s="191">
+        <f>IF(FAR!I13="","",FAR!I13)</f>
+        <v/>
+      </c>
+      <c r="G46" s="192">
+        <f>IF(FAR!K13="","",IFERROR(INDEX(FAR!$AA13:$BF13,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K13))</f>
+        <v/>
+      </c>
+      <c r="H46" s="193">
+        <f>IF(FAR!K13="",0,IF(AND(FAR!H13&lt;&gt;"",FAR!H13&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I13="",FAR!I13&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I46" s="171">
+        <f>IF($H46=1,FAR!K13,0)</f>
+        <v/>
+      </c>
+      <c r="J46" s="171">
+        <f>IF(AND(FAR!H13&lt;&gt;"",FAR!H13&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H13&lt;=ReportingFYEnd),FAR!K13,0)</f>
+        <v/>
+      </c>
+      <c r="K46" s="192">
+        <f>IF(AND(FAR!I13&lt;&gt;"",FAR!I13&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I13&lt;=ReportingFYEnd),FAR!K13,0)</f>
+        <v/>
+      </c>
+      <c r="L46" s="171">
+        <f>IF($H46=1,FAR!K13-$G46,0)</f>
+        <v/>
+      </c>
+      <c r="M46" s="171">
+        <f>IF(FAR!K13="",0,FAR!R13)</f>
+        <v/>
+      </c>
+      <c r="N46" s="193">
+        <f>IF(AND(FAR!I13&lt;&gt;"",FAR!I13&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I13&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O46" s="192">
+        <f>IF($N46=1,$L46+$M46,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="194">
+        <f>IF(FAR!K14="","",FAR!B14)</f>
+        <v/>
+      </c>
+      <c r="C47" s="195">
+        <f>IF(FAR!K14="","",FAR!C14)</f>
+        <v/>
+      </c>
+      <c r="D47" s="175">
+        <f>IF(FAR!K14="","",FAR!K14)</f>
+        <v/>
+      </c>
+      <c r="E47" s="196">
+        <f>IF(FAR!H14="","",FAR!H14)</f>
+        <v/>
+      </c>
+      <c r="F47" s="197">
+        <f>IF(FAR!I14="","",FAR!I14)</f>
+        <v/>
+      </c>
+      <c r="G47" s="198">
+        <f>IF(FAR!K14="","",IFERROR(INDEX(FAR!$AA14:$BF14,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K14))</f>
+        <v/>
+      </c>
+      <c r="H47" s="199">
+        <f>IF(FAR!K14="",0,IF(AND(FAR!H14&lt;&gt;"",FAR!H14&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I14="",FAR!I14&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I47" s="175">
+        <f>IF($H47=1,FAR!K14,0)</f>
+        <v/>
+      </c>
+      <c r="J47" s="175">
+        <f>IF(AND(FAR!H14&lt;&gt;"",FAR!H14&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H14&lt;=ReportingFYEnd),FAR!K14,0)</f>
+        <v/>
+      </c>
+      <c r="K47" s="198">
+        <f>IF(AND(FAR!I14&lt;&gt;"",FAR!I14&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I14&lt;=ReportingFYEnd),FAR!K14,0)</f>
+        <v/>
+      </c>
+      <c r="L47" s="175">
+        <f>IF($H47=1,FAR!K14-$G47,0)</f>
+        <v/>
+      </c>
+      <c r="M47" s="175">
+        <f>IF(FAR!K14="",0,FAR!R14)</f>
+        <v/>
+      </c>
+      <c r="N47" s="199">
+        <f>IF(AND(FAR!I14&lt;&gt;"",FAR!I14&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I14&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O47" s="198">
+        <f>IF($N47=1,$L47+$M47,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="188">
+        <f>IF(FAR!K15="","",FAR!B15)</f>
+        <v/>
+      </c>
+      <c r="C48" s="189">
+        <f>IF(FAR!K15="","",FAR!C15)</f>
+        <v/>
+      </c>
+      <c r="D48" s="171">
+        <f>IF(FAR!K15="","",FAR!K15)</f>
+        <v/>
+      </c>
+      <c r="E48" s="190">
+        <f>IF(FAR!H15="","",FAR!H15)</f>
+        <v/>
+      </c>
+      <c r="F48" s="191">
+        <f>IF(FAR!I15="","",FAR!I15)</f>
+        <v/>
+      </c>
+      <c r="G48" s="192">
+        <f>IF(FAR!K15="","",IFERROR(INDEX(FAR!$AA15:$BF15,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K15))</f>
+        <v/>
+      </c>
+      <c r="H48" s="193">
+        <f>IF(FAR!K15="",0,IF(AND(FAR!H15&lt;&gt;"",FAR!H15&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I15="",FAR!I15&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I48" s="171">
+        <f>IF($H48=1,FAR!K15,0)</f>
+        <v/>
+      </c>
+      <c r="J48" s="171">
+        <f>IF(AND(FAR!H15&lt;&gt;"",FAR!H15&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H15&lt;=ReportingFYEnd),FAR!K15,0)</f>
+        <v/>
+      </c>
+      <c r="K48" s="192">
+        <f>IF(AND(FAR!I15&lt;&gt;"",FAR!I15&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I15&lt;=ReportingFYEnd),FAR!K15,0)</f>
+        <v/>
+      </c>
+      <c r="L48" s="171">
+        <f>IF($H48=1,FAR!K15-$G48,0)</f>
+        <v/>
+      </c>
+      <c r="M48" s="171">
+        <f>IF(FAR!K15="",0,FAR!R15)</f>
+        <v/>
+      </c>
+      <c r="N48" s="193">
+        <f>IF(AND(FAR!I15&lt;&gt;"",FAR!I15&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I15&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O48" s="192">
+        <f>IF($N48=1,$L48+$M48,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="194">
+        <f>IF(FAR!K16="","",FAR!B16)</f>
+        <v/>
+      </c>
+      <c r="C49" s="195">
+        <f>IF(FAR!K16="","",FAR!C16)</f>
+        <v/>
+      </c>
+      <c r="D49" s="175">
+        <f>IF(FAR!K16="","",FAR!K16)</f>
+        <v/>
+      </c>
+      <c r="E49" s="196">
+        <f>IF(FAR!H16="","",FAR!H16)</f>
+        <v/>
+      </c>
+      <c r="F49" s="197">
+        <f>IF(FAR!I16="","",FAR!I16)</f>
+        <v/>
+      </c>
+      <c r="G49" s="198">
+        <f>IF(FAR!K16="","",IFERROR(INDEX(FAR!$AA16:$BF16,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K16))</f>
+        <v/>
+      </c>
+      <c r="H49" s="199">
+        <f>IF(FAR!K16="",0,IF(AND(FAR!H16&lt;&gt;"",FAR!H16&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I16="",FAR!I16&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I49" s="175">
+        <f>IF($H49=1,FAR!K16,0)</f>
+        <v/>
+      </c>
+      <c r="J49" s="175">
+        <f>IF(AND(FAR!H16&lt;&gt;"",FAR!H16&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H16&lt;=ReportingFYEnd),FAR!K16,0)</f>
+        <v/>
+      </c>
+      <c r="K49" s="198">
+        <f>IF(AND(FAR!I16&lt;&gt;"",FAR!I16&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I16&lt;=ReportingFYEnd),FAR!K16,0)</f>
+        <v/>
+      </c>
+      <c r="L49" s="175">
+        <f>IF($H49=1,FAR!K16-$G49,0)</f>
+        <v/>
+      </c>
+      <c r="M49" s="175">
+        <f>IF(FAR!K16="",0,FAR!R16)</f>
+        <v/>
+      </c>
+      <c r="N49" s="199">
+        <f>IF(AND(FAR!I16&lt;&gt;"",FAR!I16&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I16&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O49" s="198">
+        <f>IF($N49=1,$L49+$M49,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="188">
+        <f>IF(FAR!K17="","",FAR!B17)</f>
+        <v/>
+      </c>
+      <c r="C50" s="189">
+        <f>IF(FAR!K17="","",FAR!C17)</f>
+        <v/>
+      </c>
+      <c r="D50" s="171">
+        <f>IF(FAR!K17="","",FAR!K17)</f>
+        <v/>
+      </c>
+      <c r="E50" s="190">
+        <f>IF(FAR!H17="","",FAR!H17)</f>
+        <v/>
+      </c>
+      <c r="F50" s="191">
+        <f>IF(FAR!I17="","",FAR!I17)</f>
+        <v/>
+      </c>
+      <c r="G50" s="192">
+        <f>IF(FAR!K17="","",IFERROR(INDEX(FAR!$AA17:$BF17,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K17))</f>
+        <v/>
+      </c>
+      <c r="H50" s="193">
+        <f>IF(FAR!K17="",0,IF(AND(FAR!H17&lt;&gt;"",FAR!H17&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I17="",FAR!I17&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I50" s="171">
+        <f>IF($H50=1,FAR!K17,0)</f>
+        <v/>
+      </c>
+      <c r="J50" s="171">
+        <f>IF(AND(FAR!H17&lt;&gt;"",FAR!H17&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H17&lt;=ReportingFYEnd),FAR!K17,0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="192">
+        <f>IF(AND(FAR!I17&lt;&gt;"",FAR!I17&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I17&lt;=ReportingFYEnd),FAR!K17,0)</f>
+        <v/>
+      </c>
+      <c r="L50" s="171">
+        <f>IF($H50=1,FAR!K17-$G50,0)</f>
+        <v/>
+      </c>
+      <c r="M50" s="171">
+        <f>IF(FAR!K17="",0,FAR!R17)</f>
+        <v/>
+      </c>
+      <c r="N50" s="193">
+        <f>IF(AND(FAR!I17&lt;&gt;"",FAR!I17&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I17&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O50" s="192">
+        <f>IF($N50=1,$L50+$M50,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="194">
+        <f>IF(FAR!K18="","",FAR!B18)</f>
+        <v/>
+      </c>
+      <c r="C51" s="195">
+        <f>IF(FAR!K18="","",FAR!C18)</f>
+        <v/>
+      </c>
+      <c r="D51" s="175">
+        <f>IF(FAR!K18="","",FAR!K18)</f>
+        <v/>
+      </c>
+      <c r="E51" s="196">
+        <f>IF(FAR!H18="","",FAR!H18)</f>
+        <v/>
+      </c>
+      <c r="F51" s="197">
+        <f>IF(FAR!I18="","",FAR!I18)</f>
+        <v/>
+      </c>
+      <c r="G51" s="198">
+        <f>IF(FAR!K18="","",IFERROR(INDEX(FAR!$AA18:$BF18,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K18))</f>
+        <v/>
+      </c>
+      <c r="H51" s="199">
+        <f>IF(FAR!K18="",0,IF(AND(FAR!H18&lt;&gt;"",FAR!H18&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I18="",FAR!I18&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I51" s="175">
+        <f>IF($H51=1,FAR!K18,0)</f>
+        <v/>
+      </c>
+      <c r="J51" s="175">
+        <f>IF(AND(FAR!H18&lt;&gt;"",FAR!H18&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H18&lt;=ReportingFYEnd),FAR!K18,0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="198">
+        <f>IF(AND(FAR!I18&lt;&gt;"",FAR!I18&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I18&lt;=ReportingFYEnd),FAR!K18,0)</f>
+        <v/>
+      </c>
+      <c r="L51" s="175">
+        <f>IF($H51=1,FAR!K18-$G51,0)</f>
+        <v/>
+      </c>
+      <c r="M51" s="175">
+        <f>IF(FAR!K18="",0,FAR!R18)</f>
+        <v/>
+      </c>
+      <c r="N51" s="199">
+        <f>IF(AND(FAR!I18&lt;&gt;"",FAR!I18&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I18&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O51" s="198">
+        <f>IF($N51=1,$L51+$M51,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="188">
+        <f>IF(FAR!K19="","",FAR!B19)</f>
+        <v/>
+      </c>
+      <c r="C52" s="189">
+        <f>IF(FAR!K19="","",FAR!C19)</f>
+        <v/>
+      </c>
+      <c r="D52" s="171">
+        <f>IF(FAR!K19="","",FAR!K19)</f>
+        <v/>
+      </c>
+      <c r="E52" s="190">
+        <f>IF(FAR!H19="","",FAR!H19)</f>
+        <v/>
+      </c>
+      <c r="F52" s="191">
+        <f>IF(FAR!I19="","",FAR!I19)</f>
+        <v/>
+      </c>
+      <c r="G52" s="192">
+        <f>IF(FAR!K19="","",IFERROR(INDEX(FAR!$AA19:$BF19,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K19))</f>
+        <v/>
+      </c>
+      <c r="H52" s="193">
+        <f>IF(FAR!K19="",0,IF(AND(FAR!H19&lt;&gt;"",FAR!H19&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I19="",FAR!I19&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I52" s="171">
+        <f>IF($H52=1,FAR!K19,0)</f>
+        <v/>
+      </c>
+      <c r="J52" s="171">
+        <f>IF(AND(FAR!H19&lt;&gt;"",FAR!H19&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H19&lt;=ReportingFYEnd),FAR!K19,0)</f>
+        <v/>
+      </c>
+      <c r="K52" s="192">
+        <f>IF(AND(FAR!I19&lt;&gt;"",FAR!I19&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I19&lt;=ReportingFYEnd),FAR!K19,0)</f>
+        <v/>
+      </c>
+      <c r="L52" s="171">
+        <f>IF($H52=1,FAR!K19-$G52,0)</f>
+        <v/>
+      </c>
+      <c r="M52" s="171">
+        <f>IF(FAR!K19="",0,FAR!R19)</f>
+        <v/>
+      </c>
+      <c r="N52" s="193">
+        <f>IF(AND(FAR!I19&lt;&gt;"",FAR!I19&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I19&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O52" s="192">
+        <f>IF($N52=1,$L52+$M52,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="194">
+        <f>IF(FAR!K20="","",FAR!B20)</f>
+        <v/>
+      </c>
+      <c r="C53" s="195">
+        <f>IF(FAR!K20="","",FAR!C20)</f>
+        <v/>
+      </c>
+      <c r="D53" s="175">
+        <f>IF(FAR!K20="","",FAR!K20)</f>
+        <v/>
+      </c>
+      <c r="E53" s="196">
+        <f>IF(FAR!H20="","",FAR!H20)</f>
+        <v/>
+      </c>
+      <c r="F53" s="197">
+        <f>IF(FAR!I20="","",FAR!I20)</f>
+        <v/>
+      </c>
+      <c r="G53" s="198">
+        <f>IF(FAR!K20="","",IFERROR(INDEX(FAR!$AA20:$BF20,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K20))</f>
+        <v/>
+      </c>
+      <c r="H53" s="199">
+        <f>IF(FAR!K20="",0,IF(AND(FAR!H20&lt;&gt;"",FAR!H20&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I20="",FAR!I20&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I53" s="175">
+        <f>IF($H53=1,FAR!K20,0)</f>
+        <v/>
+      </c>
+      <c r="J53" s="175">
+        <f>IF(AND(FAR!H20&lt;&gt;"",FAR!H20&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H20&lt;=ReportingFYEnd),FAR!K20,0)</f>
+        <v/>
+      </c>
+      <c r="K53" s="198">
+        <f>IF(AND(FAR!I20&lt;&gt;"",FAR!I20&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I20&lt;=ReportingFYEnd),FAR!K20,0)</f>
+        <v/>
+      </c>
+      <c r="L53" s="175">
+        <f>IF($H53=1,FAR!K20-$G53,0)</f>
+        <v/>
+      </c>
+      <c r="M53" s="175">
+        <f>IF(FAR!K20="",0,FAR!R20)</f>
+        <v/>
+      </c>
+      <c r="N53" s="199">
+        <f>IF(AND(FAR!I20&lt;&gt;"",FAR!I20&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I20&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O53" s="198">
+        <f>IF($N53=1,$L53+$M53,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="188">
+        <f>IF(FAR!K21="","",FAR!B21)</f>
+        <v/>
+      </c>
+      <c r="C54" s="189">
+        <f>IF(FAR!K21="","",FAR!C21)</f>
+        <v/>
+      </c>
+      <c r="D54" s="171">
+        <f>IF(FAR!K21="","",FAR!K21)</f>
+        <v/>
+      </c>
+      <c r="E54" s="190">
+        <f>IF(FAR!H21="","",FAR!H21)</f>
+        <v/>
+      </c>
+      <c r="F54" s="191">
+        <f>IF(FAR!I21="","",FAR!I21)</f>
+        <v/>
+      </c>
+      <c r="G54" s="192">
+        <f>IF(FAR!K21="","",IFERROR(INDEX(FAR!$AA21:$BF21,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K21))</f>
+        <v/>
+      </c>
+      <c r="H54" s="193">
+        <f>IF(FAR!K21="",0,IF(AND(FAR!H21&lt;&gt;"",FAR!H21&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I21="",FAR!I21&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I54" s="171">
+        <f>IF($H54=1,FAR!K21,0)</f>
+        <v/>
+      </c>
+      <c r="J54" s="171">
+        <f>IF(AND(FAR!H21&lt;&gt;"",FAR!H21&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H21&lt;=ReportingFYEnd),FAR!K21,0)</f>
+        <v/>
+      </c>
+      <c r="K54" s="192">
+        <f>IF(AND(FAR!I21&lt;&gt;"",FAR!I21&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I21&lt;=ReportingFYEnd),FAR!K21,0)</f>
+        <v/>
+      </c>
+      <c r="L54" s="171">
+        <f>IF($H54=1,FAR!K21-$G54,0)</f>
+        <v/>
+      </c>
+      <c r="M54" s="171">
+        <f>IF(FAR!K21="",0,FAR!R21)</f>
+        <v/>
+      </c>
+      <c r="N54" s="193">
+        <f>IF(AND(FAR!I21&lt;&gt;"",FAR!I21&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I21&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O54" s="192">
+        <f>IF($N54=1,$L54+$M54,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="194">
+        <f>IF(FAR!K22="","",FAR!B22)</f>
+        <v/>
+      </c>
+      <c r="C55" s="195">
+        <f>IF(FAR!K22="","",FAR!C22)</f>
+        <v/>
+      </c>
+      <c r="D55" s="175">
+        <f>IF(FAR!K22="","",FAR!K22)</f>
+        <v/>
+      </c>
+      <c r="E55" s="196">
+        <f>IF(FAR!H22="","",FAR!H22)</f>
+        <v/>
+      </c>
+      <c r="F55" s="197">
+        <f>IF(FAR!I22="","",FAR!I22)</f>
+        <v/>
+      </c>
+      <c r="G55" s="198">
+        <f>IF(FAR!K22="","",IFERROR(INDEX(FAR!$AA22:$BF22,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K22))</f>
+        <v/>
+      </c>
+      <c r="H55" s="199">
+        <f>IF(FAR!K22="",0,IF(AND(FAR!H22&lt;&gt;"",FAR!H22&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I22="",FAR!I22&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I55" s="175">
+        <f>IF($H55=1,FAR!K22,0)</f>
+        <v/>
+      </c>
+      <c r="J55" s="175">
+        <f>IF(AND(FAR!H22&lt;&gt;"",FAR!H22&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H22&lt;=ReportingFYEnd),FAR!K22,0)</f>
+        <v/>
+      </c>
+      <c r="K55" s="198">
+        <f>IF(AND(FAR!I22&lt;&gt;"",FAR!I22&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I22&lt;=ReportingFYEnd),FAR!K22,0)</f>
+        <v/>
+      </c>
+      <c r="L55" s="175">
+        <f>IF($H55=1,FAR!K22-$G55,0)</f>
+        <v/>
+      </c>
+      <c r="M55" s="175">
+        <f>IF(FAR!K22="",0,FAR!R22)</f>
+        <v/>
+      </c>
+      <c r="N55" s="199">
+        <f>IF(AND(FAR!I22&lt;&gt;"",FAR!I22&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I22&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O55" s="198">
+        <f>IF($N55=1,$L55+$M55,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="188">
+        <f>IF(FAR!K23="","",FAR!B23)</f>
+        <v/>
+      </c>
+      <c r="C56" s="189">
+        <f>IF(FAR!K23="","",FAR!C23)</f>
+        <v/>
+      </c>
+      <c r="D56" s="171">
+        <f>IF(FAR!K23="","",FAR!K23)</f>
+        <v/>
+      </c>
+      <c r="E56" s="190">
+        <f>IF(FAR!H23="","",FAR!H23)</f>
+        <v/>
+      </c>
+      <c r="F56" s="191">
+        <f>IF(FAR!I23="","",FAR!I23)</f>
+        <v/>
+      </c>
+      <c r="G56" s="192">
+        <f>IF(FAR!K23="","",IFERROR(INDEX(FAR!$AA23:$BF23,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K23))</f>
+        <v/>
+      </c>
+      <c r="H56" s="193">
+        <f>IF(FAR!K23="",0,IF(AND(FAR!H23&lt;&gt;"",FAR!H23&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I23="",FAR!I23&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I56" s="171">
+        <f>IF($H56=1,FAR!K23,0)</f>
+        <v/>
+      </c>
+      <c r="J56" s="171">
+        <f>IF(AND(FAR!H23&lt;&gt;"",FAR!H23&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H23&lt;=ReportingFYEnd),FAR!K23,0)</f>
+        <v/>
+      </c>
+      <c r="K56" s="192">
+        <f>IF(AND(FAR!I23&lt;&gt;"",FAR!I23&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I23&lt;=ReportingFYEnd),FAR!K23,0)</f>
+        <v/>
+      </c>
+      <c r="L56" s="171">
+        <f>IF($H56=1,FAR!K23-$G56,0)</f>
+        <v/>
+      </c>
+      <c r="M56" s="171">
+        <f>IF(FAR!K23="",0,FAR!R23)</f>
+        <v/>
+      </c>
+      <c r="N56" s="193">
+        <f>IF(AND(FAR!I23&lt;&gt;"",FAR!I23&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I23&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O56" s="192">
+        <f>IF($N56=1,$L56+$M56,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="194">
+        <f>IF(FAR!K24="","",FAR!B24)</f>
+        <v/>
+      </c>
+      <c r="C57" s="195">
+        <f>IF(FAR!K24="","",FAR!C24)</f>
+        <v/>
+      </c>
+      <c r="D57" s="175">
+        <f>IF(FAR!K24="","",FAR!K24)</f>
+        <v/>
+      </c>
+      <c r="E57" s="196">
+        <f>IF(FAR!H24="","",FAR!H24)</f>
+        <v/>
+      </c>
+      <c r="F57" s="197">
+        <f>IF(FAR!I24="","",FAR!I24)</f>
+        <v/>
+      </c>
+      <c r="G57" s="198">
+        <f>IF(FAR!K24="","",IFERROR(INDEX(FAR!$AA24:$BF24,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K24))</f>
+        <v/>
+      </c>
+      <c r="H57" s="199">
+        <f>IF(FAR!K24="",0,IF(AND(FAR!H24&lt;&gt;"",FAR!H24&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I24="",FAR!I24&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I57" s="175">
+        <f>IF($H57=1,FAR!K24,0)</f>
+        <v/>
+      </c>
+      <c r="J57" s="175">
+        <f>IF(AND(FAR!H24&lt;&gt;"",FAR!H24&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H24&lt;=ReportingFYEnd),FAR!K24,0)</f>
+        <v/>
+      </c>
+      <c r="K57" s="198">
+        <f>IF(AND(FAR!I24&lt;&gt;"",FAR!I24&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I24&lt;=ReportingFYEnd),FAR!K24,0)</f>
+        <v/>
+      </c>
+      <c r="L57" s="175">
+        <f>IF($H57=1,FAR!K24-$G57,0)</f>
+        <v/>
+      </c>
+      <c r="M57" s="175">
+        <f>IF(FAR!K24="",0,FAR!R24)</f>
+        <v/>
+      </c>
+      <c r="N57" s="199">
+        <f>IF(AND(FAR!I24&lt;&gt;"",FAR!I24&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I24&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O57" s="198">
+        <f>IF($N57=1,$L57+$M57,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="188">
+        <f>IF(FAR!K25="","",FAR!B25)</f>
+        <v/>
+      </c>
+      <c r="C58" s="189">
+        <f>IF(FAR!K25="","",FAR!C25)</f>
+        <v/>
+      </c>
+      <c r="D58" s="171">
+        <f>IF(FAR!K25="","",FAR!K25)</f>
+        <v/>
+      </c>
+      <c r="E58" s="190">
+        <f>IF(FAR!H25="","",FAR!H25)</f>
+        <v/>
+      </c>
+      <c r="F58" s="191">
+        <f>IF(FAR!I25="","",FAR!I25)</f>
+        <v/>
+      </c>
+      <c r="G58" s="192">
+        <f>IF(FAR!K25="","",IFERROR(INDEX(FAR!$AA25:$BF25,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K25))</f>
+        <v/>
+      </c>
+      <c r="H58" s="193">
+        <f>IF(FAR!K25="",0,IF(AND(FAR!H25&lt;&gt;"",FAR!H25&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I25="",FAR!I25&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I58" s="171">
+        <f>IF($H58=1,FAR!K25,0)</f>
+        <v/>
+      </c>
+      <c r="J58" s="171">
+        <f>IF(AND(FAR!H25&lt;&gt;"",FAR!H25&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H25&lt;=ReportingFYEnd),FAR!K25,0)</f>
+        <v/>
+      </c>
+      <c r="K58" s="192">
+        <f>IF(AND(FAR!I25&lt;&gt;"",FAR!I25&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I25&lt;=ReportingFYEnd),FAR!K25,0)</f>
+        <v/>
+      </c>
+      <c r="L58" s="171">
+        <f>IF($H58=1,FAR!K25-$G58,0)</f>
+        <v/>
+      </c>
+      <c r="M58" s="171">
+        <f>IF(FAR!K25="",0,FAR!R25)</f>
+        <v/>
+      </c>
+      <c r="N58" s="193">
+        <f>IF(AND(FAR!I25&lt;&gt;"",FAR!I25&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I25&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O58" s="192">
+        <f>IF($N58=1,$L58+$M58,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="194">
+        <f>IF(FAR!K26="","",FAR!B26)</f>
+        <v/>
+      </c>
+      <c r="C59" s="195">
+        <f>IF(FAR!K26="","",FAR!C26)</f>
+        <v/>
+      </c>
+      <c r="D59" s="175">
+        <f>IF(FAR!K26="","",FAR!K26)</f>
+        <v/>
+      </c>
+      <c r="E59" s="196">
+        <f>IF(FAR!H26="","",FAR!H26)</f>
+        <v/>
+      </c>
+      <c r="F59" s="197">
+        <f>IF(FAR!I26="","",FAR!I26)</f>
+        <v/>
+      </c>
+      <c r="G59" s="198">
+        <f>IF(FAR!K26="","",IFERROR(INDEX(FAR!$AA26:$BF26,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K26))</f>
+        <v/>
+      </c>
+      <c r="H59" s="199">
+        <f>IF(FAR!K26="",0,IF(AND(FAR!H26&lt;&gt;"",FAR!H26&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I26="",FAR!I26&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I59" s="175">
+        <f>IF($H59=1,FAR!K26,0)</f>
+        <v/>
+      </c>
+      <c r="J59" s="175">
+        <f>IF(AND(FAR!H26&lt;&gt;"",FAR!H26&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H26&lt;=ReportingFYEnd),FAR!K26,0)</f>
+        <v/>
+      </c>
+      <c r="K59" s="198">
+        <f>IF(AND(FAR!I26&lt;&gt;"",FAR!I26&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I26&lt;=ReportingFYEnd),FAR!K26,0)</f>
+        <v/>
+      </c>
+      <c r="L59" s="175">
+        <f>IF($H59=1,FAR!K26-$G59,0)</f>
+        <v/>
+      </c>
+      <c r="M59" s="175">
+        <f>IF(FAR!K26="",0,FAR!R26)</f>
+        <v/>
+      </c>
+      <c r="N59" s="199">
+        <f>IF(AND(FAR!I26&lt;&gt;"",FAR!I26&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I26&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O59" s="198">
+        <f>IF($N59=1,$L59+$M59,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="188">
+        <f>IF(FAR!K27="","",FAR!B27)</f>
+        <v/>
+      </c>
+      <c r="C60" s="189">
+        <f>IF(FAR!K27="","",FAR!C27)</f>
+        <v/>
+      </c>
+      <c r="D60" s="171">
+        <f>IF(FAR!K27="","",FAR!K27)</f>
+        <v/>
+      </c>
+      <c r="E60" s="190">
+        <f>IF(FAR!H27="","",FAR!H27)</f>
+        <v/>
+      </c>
+      <c r="F60" s="191">
+        <f>IF(FAR!I27="","",FAR!I27)</f>
+        <v/>
+      </c>
+      <c r="G60" s="192">
+        <f>IF(FAR!K27="","",IFERROR(INDEX(FAR!$AA27:$BF27,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K27))</f>
+        <v/>
+      </c>
+      <c r="H60" s="193">
+        <f>IF(FAR!K27="",0,IF(AND(FAR!H27&lt;&gt;"",FAR!H27&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I27="",FAR!I27&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I60" s="171">
+        <f>IF($H60=1,FAR!K27,0)</f>
+        <v/>
+      </c>
+      <c r="J60" s="171">
+        <f>IF(AND(FAR!H27&lt;&gt;"",FAR!H27&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H27&lt;=ReportingFYEnd),FAR!K27,0)</f>
+        <v/>
+      </c>
+      <c r="K60" s="192">
+        <f>IF(AND(FAR!I27&lt;&gt;"",FAR!I27&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I27&lt;=ReportingFYEnd),FAR!K27,0)</f>
+        <v/>
+      </c>
+      <c r="L60" s="171">
+        <f>IF($H60=1,FAR!K27-$G60,0)</f>
+        <v/>
+      </c>
+      <c r="M60" s="171">
+        <f>IF(FAR!K27="",0,FAR!R27)</f>
+        <v/>
+      </c>
+      <c r="N60" s="193">
+        <f>IF(AND(FAR!I27&lt;&gt;"",FAR!I27&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I27&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O60" s="192">
+        <f>IF($N60=1,$L60+$M60,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="194">
+        <f>IF(FAR!K28="","",FAR!B28)</f>
+        <v/>
+      </c>
+      <c r="C61" s="195">
+        <f>IF(FAR!K28="","",FAR!C28)</f>
+        <v/>
+      </c>
+      <c r="D61" s="175">
+        <f>IF(FAR!K28="","",FAR!K28)</f>
+        <v/>
+      </c>
+      <c r="E61" s="196">
+        <f>IF(FAR!H28="","",FAR!H28)</f>
+        <v/>
+      </c>
+      <c r="F61" s="197">
+        <f>IF(FAR!I28="","",FAR!I28)</f>
+        <v/>
+      </c>
+      <c r="G61" s="198">
+        <f>IF(FAR!K28="","",IFERROR(INDEX(FAR!$AA28:$BF28,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K28))</f>
+        <v/>
+      </c>
+      <c r="H61" s="199">
+        <f>IF(FAR!K28="",0,IF(AND(FAR!H28&lt;&gt;"",FAR!H28&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I28="",FAR!I28&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I61" s="175">
+        <f>IF($H61=1,FAR!K28,0)</f>
+        <v/>
+      </c>
+      <c r="J61" s="175">
+        <f>IF(AND(FAR!H28&lt;&gt;"",FAR!H28&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H28&lt;=ReportingFYEnd),FAR!K28,0)</f>
+        <v/>
+      </c>
+      <c r="K61" s="198">
+        <f>IF(AND(FAR!I28&lt;&gt;"",FAR!I28&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I28&lt;=ReportingFYEnd),FAR!K28,0)</f>
+        <v/>
+      </c>
+      <c r="L61" s="175">
+        <f>IF($H61=1,FAR!K28-$G61,0)</f>
+        <v/>
+      </c>
+      <c r="M61" s="175">
+        <f>IF(FAR!K28="",0,FAR!R28)</f>
+        <v/>
+      </c>
+      <c r="N61" s="199">
+        <f>IF(AND(FAR!I28&lt;&gt;"",FAR!I28&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I28&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O61" s="198">
+        <f>IF($N61=1,$L61+$M61,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="188">
+        <f>IF(FAR!K29="","",FAR!B29)</f>
+        <v/>
+      </c>
+      <c r="C62" s="189">
+        <f>IF(FAR!K29="","",FAR!C29)</f>
+        <v/>
+      </c>
+      <c r="D62" s="171">
+        <f>IF(FAR!K29="","",FAR!K29)</f>
+        <v/>
+      </c>
+      <c r="E62" s="190">
+        <f>IF(FAR!H29="","",FAR!H29)</f>
+        <v/>
+      </c>
+      <c r="F62" s="191">
+        <f>IF(FAR!I29="","",FAR!I29)</f>
+        <v/>
+      </c>
+      <c r="G62" s="192">
+        <f>IF(FAR!K29="","",IFERROR(INDEX(FAR!$AA29:$BF29,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K29))</f>
+        <v/>
+      </c>
+      <c r="H62" s="193">
+        <f>IF(FAR!K29="",0,IF(AND(FAR!H29&lt;&gt;"",FAR!H29&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I29="",FAR!I29&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I62" s="171">
+        <f>IF($H62=1,FAR!K29,0)</f>
+        <v/>
+      </c>
+      <c r="J62" s="171">
+        <f>IF(AND(FAR!H29&lt;&gt;"",FAR!H29&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H29&lt;=ReportingFYEnd),FAR!K29,0)</f>
+        <v/>
+      </c>
+      <c r="K62" s="192">
+        <f>IF(AND(FAR!I29&lt;&gt;"",FAR!I29&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I29&lt;=ReportingFYEnd),FAR!K29,0)</f>
+        <v/>
+      </c>
+      <c r="L62" s="171">
+        <f>IF($H62=1,FAR!K29-$G62,0)</f>
+        <v/>
+      </c>
+      <c r="M62" s="171">
+        <f>IF(FAR!K29="",0,FAR!R29)</f>
+        <v/>
+      </c>
+      <c r="N62" s="193">
+        <f>IF(AND(FAR!I29&lt;&gt;"",FAR!I29&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I29&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O62" s="192">
+        <f>IF($N62=1,$L62+$M62,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="194">
+        <f>IF(FAR!K30="","",FAR!B30)</f>
+        <v/>
+      </c>
+      <c r="C63" s="195">
+        <f>IF(FAR!K30="","",FAR!C30)</f>
+        <v/>
+      </c>
+      <c r="D63" s="175">
+        <f>IF(FAR!K30="","",FAR!K30)</f>
+        <v/>
+      </c>
+      <c r="E63" s="196">
+        <f>IF(FAR!H30="","",FAR!H30)</f>
+        <v/>
+      </c>
+      <c r="F63" s="197">
+        <f>IF(FAR!I30="","",FAR!I30)</f>
+        <v/>
+      </c>
+      <c r="G63" s="198">
+        <f>IF(FAR!K30="","",IFERROR(INDEX(FAR!$AA30:$BF30,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K30))</f>
+        <v/>
+      </c>
+      <c r="H63" s="199">
+        <f>IF(FAR!K30="",0,IF(AND(FAR!H30&lt;&gt;"",FAR!H30&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I30="",FAR!I30&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I63" s="175">
+        <f>IF($H63=1,FAR!K30,0)</f>
+        <v/>
+      </c>
+      <c r="J63" s="175">
+        <f>IF(AND(FAR!H30&lt;&gt;"",FAR!H30&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H30&lt;=ReportingFYEnd),FAR!K30,0)</f>
+        <v/>
+      </c>
+      <c r="K63" s="198">
+        <f>IF(AND(FAR!I30&lt;&gt;"",FAR!I30&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I30&lt;=ReportingFYEnd),FAR!K30,0)</f>
+        <v/>
+      </c>
+      <c r="L63" s="175">
+        <f>IF($H63=1,FAR!K30-$G63,0)</f>
+        <v/>
+      </c>
+      <c r="M63" s="175">
+        <f>IF(FAR!K30="",0,FAR!R30)</f>
+        <v/>
+      </c>
+      <c r="N63" s="199">
+        <f>IF(AND(FAR!I30&lt;&gt;"",FAR!I30&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I30&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O63" s="198">
+        <f>IF($N63=1,$L63+$M63,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="188">
+        <f>IF(FAR!K31="","",FAR!B31)</f>
+        <v/>
+      </c>
+      <c r="C64" s="189">
+        <f>IF(FAR!K31="","",FAR!C31)</f>
+        <v/>
+      </c>
+      <c r="D64" s="171">
+        <f>IF(FAR!K31="","",FAR!K31)</f>
+        <v/>
+      </c>
+      <c r="E64" s="190">
+        <f>IF(FAR!H31="","",FAR!H31)</f>
+        <v/>
+      </c>
+      <c r="F64" s="191">
+        <f>IF(FAR!I31="","",FAR!I31)</f>
+        <v/>
+      </c>
+      <c r="G64" s="192">
+        <f>IF(FAR!K31="","",IFERROR(INDEX(FAR!$AA31:$BF31,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K31))</f>
+        <v/>
+      </c>
+      <c r="H64" s="193">
+        <f>IF(FAR!K31="",0,IF(AND(FAR!H31&lt;&gt;"",FAR!H31&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I31="",FAR!I31&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I64" s="171">
+        <f>IF($H64=1,FAR!K31,0)</f>
+        <v/>
+      </c>
+      <c r="J64" s="171">
+        <f>IF(AND(FAR!H31&lt;&gt;"",FAR!H31&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H31&lt;=ReportingFYEnd),FAR!K31,0)</f>
+        <v/>
+      </c>
+      <c r="K64" s="192">
+        <f>IF(AND(FAR!I31&lt;&gt;"",FAR!I31&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I31&lt;=ReportingFYEnd),FAR!K31,0)</f>
+        <v/>
+      </c>
+      <c r="L64" s="171">
+        <f>IF($H64=1,FAR!K31-$G64,0)</f>
+        <v/>
+      </c>
+      <c r="M64" s="171">
+        <f>IF(FAR!K31="",0,FAR!R31)</f>
+        <v/>
+      </c>
+      <c r="N64" s="193">
+        <f>IF(AND(FAR!I31&lt;&gt;"",FAR!I31&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I31&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O64" s="192">
+        <f>IF($N64=1,$L64+$M64,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="194">
+        <f>IF(FAR!K32="","",FAR!B32)</f>
+        <v/>
+      </c>
+      <c r="C65" s="195">
+        <f>IF(FAR!K32="","",FAR!C32)</f>
+        <v/>
+      </c>
+      <c r="D65" s="175">
+        <f>IF(FAR!K32="","",FAR!K32)</f>
+        <v/>
+      </c>
+      <c r="E65" s="196">
+        <f>IF(FAR!H32="","",FAR!H32)</f>
+        <v/>
+      </c>
+      <c r="F65" s="197">
+        <f>IF(FAR!I32="","",FAR!I32)</f>
+        <v/>
+      </c>
+      <c r="G65" s="198">
+        <f>IF(FAR!K32="","",IFERROR(INDEX(FAR!$AA32:$BF32,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K32))</f>
+        <v/>
+      </c>
+      <c r="H65" s="199">
+        <f>IF(FAR!K32="",0,IF(AND(FAR!H32&lt;&gt;"",FAR!H32&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I32="",FAR!I32&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I65" s="175">
+        <f>IF($H65=1,FAR!K32,0)</f>
+        <v/>
+      </c>
+      <c r="J65" s="175">
+        <f>IF(AND(FAR!H32&lt;&gt;"",FAR!H32&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H32&lt;=ReportingFYEnd),FAR!K32,0)</f>
+        <v/>
+      </c>
+      <c r="K65" s="198">
+        <f>IF(AND(FAR!I32&lt;&gt;"",FAR!I32&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I32&lt;=ReportingFYEnd),FAR!K32,0)</f>
+        <v/>
+      </c>
+      <c r="L65" s="175">
+        <f>IF($H65=1,FAR!K32-$G65,0)</f>
+        <v/>
+      </c>
+      <c r="M65" s="175">
+        <f>IF(FAR!K32="",0,FAR!R32)</f>
+        <v/>
+      </c>
+      <c r="N65" s="199">
+        <f>IF(AND(FAR!I32&lt;&gt;"",FAR!I32&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I32&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O65" s="198">
+        <f>IF($N65=1,$L65+$M65,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="188">
+        <f>IF(FAR!K33="","",FAR!B33)</f>
+        <v/>
+      </c>
+      <c r="C66" s="189">
+        <f>IF(FAR!K33="","",FAR!C33)</f>
+        <v/>
+      </c>
+      <c r="D66" s="171">
+        <f>IF(FAR!K33="","",FAR!K33)</f>
+        <v/>
+      </c>
+      <c r="E66" s="190">
+        <f>IF(FAR!H33="","",FAR!H33)</f>
+        <v/>
+      </c>
+      <c r="F66" s="191">
+        <f>IF(FAR!I33="","",FAR!I33)</f>
+        <v/>
+      </c>
+      <c r="G66" s="192">
+        <f>IF(FAR!K33="","",IFERROR(INDEX(FAR!$AA33:$BF33,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K33))</f>
+        <v/>
+      </c>
+      <c r="H66" s="193">
+        <f>IF(FAR!K33="",0,IF(AND(FAR!H33&lt;&gt;"",FAR!H33&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I33="",FAR!I33&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I66" s="171">
+        <f>IF($H66=1,FAR!K33,0)</f>
+        <v/>
+      </c>
+      <c r="J66" s="171">
+        <f>IF(AND(FAR!H33&lt;&gt;"",FAR!H33&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H33&lt;=ReportingFYEnd),FAR!K33,0)</f>
+        <v/>
+      </c>
+      <c r="K66" s="192">
+        <f>IF(AND(FAR!I33&lt;&gt;"",FAR!I33&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I33&lt;=ReportingFYEnd),FAR!K33,0)</f>
+        <v/>
+      </c>
+      <c r="L66" s="171">
+        <f>IF($H66=1,FAR!K33-$G66,0)</f>
+        <v/>
+      </c>
+      <c r="M66" s="171">
+        <f>IF(FAR!K33="",0,FAR!R33)</f>
+        <v/>
+      </c>
+      <c r="N66" s="193">
+        <f>IF(AND(FAR!I33&lt;&gt;"",FAR!I33&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I33&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O66" s="192">
+        <f>IF($N66=1,$L66+$M66,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="194">
+        <f>IF(FAR!K34="","",FAR!B34)</f>
+        <v/>
+      </c>
+      <c r="C67" s="195">
+        <f>IF(FAR!K34="","",FAR!C34)</f>
+        <v/>
+      </c>
+      <c r="D67" s="175">
+        <f>IF(FAR!K34="","",FAR!K34)</f>
+        <v/>
+      </c>
+      <c r="E67" s="196">
+        <f>IF(FAR!H34="","",FAR!H34)</f>
+        <v/>
+      </c>
+      <c r="F67" s="197">
+        <f>IF(FAR!I34="","",FAR!I34)</f>
+        <v/>
+      </c>
+      <c r="G67" s="198">
+        <f>IF(FAR!K34="","",IFERROR(INDEX(FAR!$AA34:$BF34,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K34))</f>
+        <v/>
+      </c>
+      <c r="H67" s="199">
+        <f>IF(FAR!K34="",0,IF(AND(FAR!H34&lt;&gt;"",FAR!H34&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I34="",FAR!I34&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I67" s="175">
+        <f>IF($H67=1,FAR!K34,0)</f>
+        <v/>
+      </c>
+      <c r="J67" s="175">
+        <f>IF(AND(FAR!H34&lt;&gt;"",FAR!H34&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H34&lt;=ReportingFYEnd),FAR!K34,0)</f>
+        <v/>
+      </c>
+      <c r="K67" s="198">
+        <f>IF(AND(FAR!I34&lt;&gt;"",FAR!I34&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I34&lt;=ReportingFYEnd),FAR!K34,0)</f>
+        <v/>
+      </c>
+      <c r="L67" s="175">
+        <f>IF($H67=1,FAR!K34-$G67,0)</f>
+        <v/>
+      </c>
+      <c r="M67" s="175">
+        <f>IF(FAR!K34="",0,FAR!R34)</f>
+        <v/>
+      </c>
+      <c r="N67" s="199">
+        <f>IF(AND(FAR!I34&lt;&gt;"",FAR!I34&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I34&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O67" s="198">
+        <f>IF($N67=1,$L67+$M67,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="188">
+        <f>IF(FAR!K35="","",FAR!B35)</f>
+        <v/>
+      </c>
+      <c r="C68" s="189">
+        <f>IF(FAR!K35="","",FAR!C35)</f>
+        <v/>
+      </c>
+      <c r="D68" s="171">
+        <f>IF(FAR!K35="","",FAR!K35)</f>
+        <v/>
+      </c>
+      <c r="E68" s="190">
+        <f>IF(FAR!H35="","",FAR!H35)</f>
+        <v/>
+      </c>
+      <c r="F68" s="191">
+        <f>IF(FAR!I35="","",FAR!I35)</f>
+        <v/>
+      </c>
+      <c r="G68" s="192">
+        <f>IF(FAR!K35="","",IFERROR(INDEX(FAR!$AA35:$BF35,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K35))</f>
+        <v/>
+      </c>
+      <c r="H68" s="193">
+        <f>IF(FAR!K35="",0,IF(AND(FAR!H35&lt;&gt;"",FAR!H35&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I35="",FAR!I35&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I68" s="171">
+        <f>IF($H68=1,FAR!K35,0)</f>
+        <v/>
+      </c>
+      <c r="J68" s="171">
+        <f>IF(AND(FAR!H35&lt;&gt;"",FAR!H35&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H35&lt;=ReportingFYEnd),FAR!K35,0)</f>
+        <v/>
+      </c>
+      <c r="K68" s="192">
+        <f>IF(AND(FAR!I35&lt;&gt;"",FAR!I35&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I35&lt;=ReportingFYEnd),FAR!K35,0)</f>
+        <v/>
+      </c>
+      <c r="L68" s="171">
+        <f>IF($H68=1,FAR!K35-$G68,0)</f>
+        <v/>
+      </c>
+      <c r="M68" s="171">
+        <f>IF(FAR!K35="",0,FAR!R35)</f>
+        <v/>
+      </c>
+      <c r="N68" s="193">
+        <f>IF(AND(FAR!I35&lt;&gt;"",FAR!I35&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I35&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O68" s="192">
+        <f>IF($N68=1,$L68+$M68,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="194">
+        <f>IF(FAR!K36="","",FAR!B36)</f>
+        <v/>
+      </c>
+      <c r="C69" s="195">
+        <f>IF(FAR!K36="","",FAR!C36)</f>
+        <v/>
+      </c>
+      <c r="D69" s="175">
+        <f>IF(FAR!K36="","",FAR!K36)</f>
+        <v/>
+      </c>
+      <c r="E69" s="196">
+        <f>IF(FAR!H36="","",FAR!H36)</f>
+        <v/>
+      </c>
+      <c r="F69" s="197">
+        <f>IF(FAR!I36="","",FAR!I36)</f>
+        <v/>
+      </c>
+      <c r="G69" s="198">
+        <f>IF(FAR!K36="","",IFERROR(INDEX(FAR!$AA36:$BF36,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K36))</f>
+        <v/>
+      </c>
+      <c r="H69" s="199">
+        <f>IF(FAR!K36="",0,IF(AND(FAR!H36&lt;&gt;"",FAR!H36&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I36="",FAR!I36&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I69" s="175">
+        <f>IF($H69=1,FAR!K36,0)</f>
+        <v/>
+      </c>
+      <c r="J69" s="175">
+        <f>IF(AND(FAR!H36&lt;&gt;"",FAR!H36&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H36&lt;=ReportingFYEnd),FAR!K36,0)</f>
+        <v/>
+      </c>
+      <c r="K69" s="198">
+        <f>IF(AND(FAR!I36&lt;&gt;"",FAR!I36&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I36&lt;=ReportingFYEnd),FAR!K36,0)</f>
+        <v/>
+      </c>
+      <c r="L69" s="175">
+        <f>IF($H69=1,FAR!K36-$G69,0)</f>
+        <v/>
+      </c>
+      <c r="M69" s="175">
+        <f>IF(FAR!K36="",0,FAR!R36)</f>
+        <v/>
+      </c>
+      <c r="N69" s="199">
+        <f>IF(AND(FAR!I36&lt;&gt;"",FAR!I36&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I36&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O69" s="198">
+        <f>IF($N69=1,$L69+$M69,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="188">
+        <f>IF(FAR!K37="","",FAR!B37)</f>
+        <v/>
+      </c>
+      <c r="C70" s="189">
+        <f>IF(FAR!K37="","",FAR!C37)</f>
+        <v/>
+      </c>
+      <c r="D70" s="171">
+        <f>IF(FAR!K37="","",FAR!K37)</f>
+        <v/>
+      </c>
+      <c r="E70" s="190">
+        <f>IF(FAR!H37="","",FAR!H37)</f>
+        <v/>
+      </c>
+      <c r="F70" s="191">
+        <f>IF(FAR!I37="","",FAR!I37)</f>
+        <v/>
+      </c>
+      <c r="G70" s="192">
+        <f>IF(FAR!K37="","",IFERROR(INDEX(FAR!$AA37:$BF37,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K37))</f>
+        <v/>
+      </c>
+      <c r="H70" s="193">
+        <f>IF(FAR!K37="",0,IF(AND(FAR!H37&lt;&gt;"",FAR!H37&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I37="",FAR!I37&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I70" s="171">
+        <f>IF($H70=1,FAR!K37,0)</f>
+        <v/>
+      </c>
+      <c r="J70" s="171">
+        <f>IF(AND(FAR!H37&lt;&gt;"",FAR!H37&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H37&lt;=ReportingFYEnd),FAR!K37,0)</f>
+        <v/>
+      </c>
+      <c r="K70" s="192">
+        <f>IF(AND(FAR!I37&lt;&gt;"",FAR!I37&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I37&lt;=ReportingFYEnd),FAR!K37,0)</f>
+        <v/>
+      </c>
+      <c r="L70" s="171">
+        <f>IF($H70=1,FAR!K37-$G70,0)</f>
+        <v/>
+      </c>
+      <c r="M70" s="171">
+        <f>IF(FAR!K37="",0,FAR!R37)</f>
+        <v/>
+      </c>
+      <c r="N70" s="193">
+        <f>IF(AND(FAR!I37&lt;&gt;"",FAR!I37&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I37&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O70" s="192">
+        <f>IF($N70=1,$L70+$M70,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="194">
+        <f>IF(FAR!K38="","",FAR!B38)</f>
+        <v/>
+      </c>
+      <c r="C71" s="195">
+        <f>IF(FAR!K38="","",FAR!C38)</f>
+        <v/>
+      </c>
+      <c r="D71" s="175">
+        <f>IF(FAR!K38="","",FAR!K38)</f>
+        <v/>
+      </c>
+      <c r="E71" s="196">
+        <f>IF(FAR!H38="","",FAR!H38)</f>
+        <v/>
+      </c>
+      <c r="F71" s="197">
+        <f>IF(FAR!I38="","",FAR!I38)</f>
+        <v/>
+      </c>
+      <c r="G71" s="198">
+        <f>IF(FAR!K38="","",IFERROR(INDEX(FAR!$AA38:$BF38,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K38))</f>
+        <v/>
+      </c>
+      <c r="H71" s="199">
+        <f>IF(FAR!K38="",0,IF(AND(FAR!H38&lt;&gt;"",FAR!H38&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I38="",FAR!I38&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I71" s="175">
+        <f>IF($H71=1,FAR!K38,0)</f>
+        <v/>
+      </c>
+      <c r="J71" s="175">
+        <f>IF(AND(FAR!H38&lt;&gt;"",FAR!H38&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H38&lt;=ReportingFYEnd),FAR!K38,0)</f>
+        <v/>
+      </c>
+      <c r="K71" s="198">
+        <f>IF(AND(FAR!I38&lt;&gt;"",FAR!I38&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I38&lt;=ReportingFYEnd),FAR!K38,0)</f>
+        <v/>
+      </c>
+      <c r="L71" s="175">
+        <f>IF($H71=1,FAR!K38-$G71,0)</f>
+        <v/>
+      </c>
+      <c r="M71" s="175">
+        <f>IF(FAR!K38="",0,FAR!R38)</f>
+        <v/>
+      </c>
+      <c r="N71" s="199">
+        <f>IF(AND(FAR!I38&lt;&gt;"",FAR!I38&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I38&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O71" s="198">
+        <f>IF($N71=1,$L71+$M71,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="188">
+        <f>IF(FAR!K39="","",FAR!B39)</f>
+        <v/>
+      </c>
+      <c r="C72" s="189">
+        <f>IF(FAR!K39="","",FAR!C39)</f>
+        <v/>
+      </c>
+      <c r="D72" s="171">
+        <f>IF(FAR!K39="","",FAR!K39)</f>
+        <v/>
+      </c>
+      <c r="E72" s="190">
+        <f>IF(FAR!H39="","",FAR!H39)</f>
+        <v/>
+      </c>
+      <c r="F72" s="191">
+        <f>IF(FAR!I39="","",FAR!I39)</f>
+        <v/>
+      </c>
+      <c r="G72" s="192">
+        <f>IF(FAR!K39="","",IFERROR(INDEX(FAR!$AA39:$BF39,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K39))</f>
+        <v/>
+      </c>
+      <c r="H72" s="193">
+        <f>IF(FAR!K39="",0,IF(AND(FAR!H39&lt;&gt;"",FAR!H39&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I39="",FAR!I39&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I72" s="171">
+        <f>IF($H72=1,FAR!K39,0)</f>
+        <v/>
+      </c>
+      <c r="J72" s="171">
+        <f>IF(AND(FAR!H39&lt;&gt;"",FAR!H39&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H39&lt;=ReportingFYEnd),FAR!K39,0)</f>
+        <v/>
+      </c>
+      <c r="K72" s="192">
+        <f>IF(AND(FAR!I39&lt;&gt;"",FAR!I39&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I39&lt;=ReportingFYEnd),FAR!K39,0)</f>
+        <v/>
+      </c>
+      <c r="L72" s="171">
+        <f>IF($H72=1,FAR!K39-$G72,0)</f>
+        <v/>
+      </c>
+      <c r="M72" s="171">
+        <f>IF(FAR!K39="",0,FAR!R39)</f>
+        <v/>
+      </c>
+      <c r="N72" s="193">
+        <f>IF(AND(FAR!I39&lt;&gt;"",FAR!I39&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I39&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O72" s="192">
+        <f>IF($N72=1,$L72+$M72,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="194">
+        <f>IF(FAR!K40="","",FAR!B40)</f>
+        <v/>
+      </c>
+      <c r="C73" s="195">
+        <f>IF(FAR!K40="","",FAR!C40)</f>
+        <v/>
+      </c>
+      <c r="D73" s="175">
+        <f>IF(FAR!K40="","",FAR!K40)</f>
+        <v/>
+      </c>
+      <c r="E73" s="196">
+        <f>IF(FAR!H40="","",FAR!H40)</f>
+        <v/>
+      </c>
+      <c r="F73" s="197">
+        <f>IF(FAR!I40="","",FAR!I40)</f>
+        <v/>
+      </c>
+      <c r="G73" s="198">
+        <f>IF(FAR!K40="","",IFERROR(INDEX(FAR!$AA40:$BF40,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K40))</f>
+        <v/>
+      </c>
+      <c r="H73" s="199">
+        <f>IF(FAR!K40="",0,IF(AND(FAR!H40&lt;&gt;"",FAR!H40&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I40="",FAR!I40&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I73" s="175">
+        <f>IF($H73=1,FAR!K40,0)</f>
+        <v/>
+      </c>
+      <c r="J73" s="175">
+        <f>IF(AND(FAR!H40&lt;&gt;"",FAR!H40&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H40&lt;=ReportingFYEnd),FAR!K40,0)</f>
+        <v/>
+      </c>
+      <c r="K73" s="198">
+        <f>IF(AND(FAR!I40&lt;&gt;"",FAR!I40&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I40&lt;=ReportingFYEnd),FAR!K40,0)</f>
+        <v/>
+      </c>
+      <c r="L73" s="175">
+        <f>IF($H73=1,FAR!K40-$G73,0)</f>
+        <v/>
+      </c>
+      <c r="M73" s="175">
+        <f>IF(FAR!K40="",0,FAR!R40)</f>
+        <v/>
+      </c>
+      <c r="N73" s="199">
+        <f>IF(AND(FAR!I40&lt;&gt;"",FAR!I40&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I40&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O73" s="198">
+        <f>IF($N73=1,$L73+$M73,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="188">
+        <f>IF(FAR!K41="","",FAR!B41)</f>
+        <v/>
+      </c>
+      <c r="C74" s="189">
+        <f>IF(FAR!K41="","",FAR!C41)</f>
+        <v/>
+      </c>
+      <c r="D74" s="171">
+        <f>IF(FAR!K41="","",FAR!K41)</f>
+        <v/>
+      </c>
+      <c r="E74" s="190">
+        <f>IF(FAR!H41="","",FAR!H41)</f>
+        <v/>
+      </c>
+      <c r="F74" s="191">
+        <f>IF(FAR!I41="","",FAR!I41)</f>
+        <v/>
+      </c>
+      <c r="G74" s="192">
+        <f>IF(FAR!K41="","",IFERROR(INDEX(FAR!$AA41:$BF41,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K41))</f>
+        <v/>
+      </c>
+      <c r="H74" s="193">
+        <f>IF(FAR!K41="",0,IF(AND(FAR!H41&lt;&gt;"",FAR!H41&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I41="",FAR!I41&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I74" s="171">
+        <f>IF($H74=1,FAR!K41,0)</f>
+        <v/>
+      </c>
+      <c r="J74" s="171">
+        <f>IF(AND(FAR!H41&lt;&gt;"",FAR!H41&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H41&lt;=ReportingFYEnd),FAR!K41,0)</f>
+        <v/>
+      </c>
+      <c r="K74" s="192">
+        <f>IF(AND(FAR!I41&lt;&gt;"",FAR!I41&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I41&lt;=ReportingFYEnd),FAR!K41,0)</f>
+        <v/>
+      </c>
+      <c r="L74" s="171">
+        <f>IF($H74=1,FAR!K41-$G74,0)</f>
+        <v/>
+      </c>
+      <c r="M74" s="171">
+        <f>IF(FAR!K41="",0,FAR!R41)</f>
+        <v/>
+      </c>
+      <c r="N74" s="193">
+        <f>IF(AND(FAR!I41&lt;&gt;"",FAR!I41&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I41&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O74" s="192">
+        <f>IF($N74=1,$L74+$M74,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="194">
+        <f>IF(FAR!K42="","",FAR!B42)</f>
+        <v/>
+      </c>
+      <c r="C75" s="195">
+        <f>IF(FAR!K42="","",FAR!C42)</f>
+        <v/>
+      </c>
+      <c r="D75" s="175">
+        <f>IF(FAR!K42="","",FAR!K42)</f>
+        <v/>
+      </c>
+      <c r="E75" s="196">
+        <f>IF(FAR!H42="","",FAR!H42)</f>
+        <v/>
+      </c>
+      <c r="F75" s="197">
+        <f>IF(FAR!I42="","",FAR!I42)</f>
+        <v/>
+      </c>
+      <c r="G75" s="198">
+        <f>IF(FAR!K42="","",IFERROR(INDEX(FAR!$AA42:$BF42,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K42))</f>
+        <v/>
+      </c>
+      <c r="H75" s="199">
+        <f>IF(FAR!K42="",0,IF(AND(FAR!H42&lt;&gt;"",FAR!H42&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I42="",FAR!I42&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I75" s="175">
+        <f>IF($H75=1,FAR!K42,0)</f>
+        <v/>
+      </c>
+      <c r="J75" s="175">
+        <f>IF(AND(FAR!H42&lt;&gt;"",FAR!H42&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H42&lt;=ReportingFYEnd),FAR!K42,0)</f>
+        <v/>
+      </c>
+      <c r="K75" s="198">
+        <f>IF(AND(FAR!I42&lt;&gt;"",FAR!I42&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I42&lt;=ReportingFYEnd),FAR!K42,0)</f>
+        <v/>
+      </c>
+      <c r="L75" s="175">
+        <f>IF($H75=1,FAR!K42-$G75,0)</f>
+        <v/>
+      </c>
+      <c r="M75" s="175">
+        <f>IF(FAR!K42="",0,FAR!R42)</f>
+        <v/>
+      </c>
+      <c r="N75" s="199">
+        <f>IF(AND(FAR!I42&lt;&gt;"",FAR!I42&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I42&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O75" s="198">
+        <f>IF($N75=1,$L75+$M75,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="188">
+        <f>IF(FAR!K43="","",FAR!B43)</f>
+        <v/>
+      </c>
+      <c r="C76" s="189">
+        <f>IF(FAR!K43="","",FAR!C43)</f>
+        <v/>
+      </c>
+      <c r="D76" s="171">
+        <f>IF(FAR!K43="","",FAR!K43)</f>
+        <v/>
+      </c>
+      <c r="E76" s="190">
+        <f>IF(FAR!H43="","",FAR!H43)</f>
+        <v/>
+      </c>
+      <c r="F76" s="191">
+        <f>IF(FAR!I43="","",FAR!I43)</f>
+        <v/>
+      </c>
+      <c r="G76" s="192">
+        <f>IF(FAR!K43="","",IFERROR(INDEX(FAR!$AA43:$BF43,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K43))</f>
+        <v/>
+      </c>
+      <c r="H76" s="193">
+        <f>IF(FAR!K43="",0,IF(AND(FAR!H43&lt;&gt;"",FAR!H43&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I43="",FAR!I43&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I76" s="171">
+        <f>IF($H76=1,FAR!K43,0)</f>
+        <v/>
+      </c>
+      <c r="J76" s="171">
+        <f>IF(AND(FAR!H43&lt;&gt;"",FAR!H43&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H43&lt;=ReportingFYEnd),FAR!K43,0)</f>
+        <v/>
+      </c>
+      <c r="K76" s="192">
+        <f>IF(AND(FAR!I43&lt;&gt;"",FAR!I43&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I43&lt;=ReportingFYEnd),FAR!K43,0)</f>
+        <v/>
+      </c>
+      <c r="L76" s="171">
+        <f>IF($H76=1,FAR!K43-$G76,0)</f>
+        <v/>
+      </c>
+      <c r="M76" s="171">
+        <f>IF(FAR!K43="",0,FAR!R43)</f>
+        <v/>
+      </c>
+      <c r="N76" s="193">
+        <f>IF(AND(FAR!I43&lt;&gt;"",FAR!I43&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I43&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O76" s="192">
+        <f>IF($N76=1,$L76+$M76,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="194">
+        <f>IF(FAR!K44="","",FAR!B44)</f>
+        <v/>
+      </c>
+      <c r="C77" s="195">
+        <f>IF(FAR!K44="","",FAR!C44)</f>
+        <v/>
+      </c>
+      <c r="D77" s="175">
+        <f>IF(FAR!K44="","",FAR!K44)</f>
+        <v/>
+      </c>
+      <c r="E77" s="196">
+        <f>IF(FAR!H44="","",FAR!H44)</f>
+        <v/>
+      </c>
+      <c r="F77" s="197">
+        <f>IF(FAR!I44="","",FAR!I44)</f>
+        <v/>
+      </c>
+      <c r="G77" s="198">
+        <f>IF(FAR!K44="","",IFERROR(INDEX(FAR!$AA44:$BF44,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K44))</f>
+        <v/>
+      </c>
+      <c r="H77" s="199">
+        <f>IF(FAR!K44="",0,IF(AND(FAR!H44&lt;&gt;"",FAR!H44&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I44="",FAR!I44&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I77" s="175">
+        <f>IF($H77=1,FAR!K44,0)</f>
+        <v/>
+      </c>
+      <c r="J77" s="175">
+        <f>IF(AND(FAR!H44&lt;&gt;"",FAR!H44&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H44&lt;=ReportingFYEnd),FAR!K44,0)</f>
+        <v/>
+      </c>
+      <c r="K77" s="198">
+        <f>IF(AND(FAR!I44&lt;&gt;"",FAR!I44&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I44&lt;=ReportingFYEnd),FAR!K44,0)</f>
+        <v/>
+      </c>
+      <c r="L77" s="175">
+        <f>IF($H77=1,FAR!K44-$G77,0)</f>
+        <v/>
+      </c>
+      <c r="M77" s="175">
+        <f>IF(FAR!K44="",0,FAR!R44)</f>
+        <v/>
+      </c>
+      <c r="N77" s="199">
+        <f>IF(AND(FAR!I44&lt;&gt;"",FAR!I44&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I44&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O77" s="198">
+        <f>IF($N77=1,$L77+$M77,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="188">
+        <f>IF(FAR!K45="","",FAR!B45)</f>
+        <v/>
+      </c>
+      <c r="C78" s="189">
+        <f>IF(FAR!K45="","",FAR!C45)</f>
+        <v/>
+      </c>
+      <c r="D78" s="171">
+        <f>IF(FAR!K45="","",FAR!K45)</f>
+        <v/>
+      </c>
+      <c r="E78" s="190">
+        <f>IF(FAR!H45="","",FAR!H45)</f>
+        <v/>
+      </c>
+      <c r="F78" s="191">
+        <f>IF(FAR!I45="","",FAR!I45)</f>
+        <v/>
+      </c>
+      <c r="G78" s="192">
+        <f>IF(FAR!K45="","",IFERROR(INDEX(FAR!$AA45:$BF45,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K45))</f>
+        <v/>
+      </c>
+      <c r="H78" s="193">
+        <f>IF(FAR!K45="",0,IF(AND(FAR!H45&lt;&gt;"",FAR!H45&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I45="",FAR!I45&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I78" s="171">
+        <f>IF($H78=1,FAR!K45,0)</f>
+        <v/>
+      </c>
+      <c r="J78" s="171">
+        <f>IF(AND(FAR!H45&lt;&gt;"",FAR!H45&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H45&lt;=ReportingFYEnd),FAR!K45,0)</f>
+        <v/>
+      </c>
+      <c r="K78" s="192">
+        <f>IF(AND(FAR!I45&lt;&gt;"",FAR!I45&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I45&lt;=ReportingFYEnd),FAR!K45,0)</f>
+        <v/>
+      </c>
+      <c r="L78" s="171">
+        <f>IF($H78=1,FAR!K45-$G78,0)</f>
+        <v/>
+      </c>
+      <c r="M78" s="171">
+        <f>IF(FAR!K45="",0,FAR!R45)</f>
+        <v/>
+      </c>
+      <c r="N78" s="193">
+        <f>IF(AND(FAR!I45&lt;&gt;"",FAR!I45&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I45&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O78" s="192">
+        <f>IF($N78=1,$L78+$M78,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="194">
+        <f>IF(FAR!K46="","",FAR!B46)</f>
+        <v/>
+      </c>
+      <c r="C79" s="195">
+        <f>IF(FAR!K46="","",FAR!C46)</f>
+        <v/>
+      </c>
+      <c r="D79" s="175">
+        <f>IF(FAR!K46="","",FAR!K46)</f>
+        <v/>
+      </c>
+      <c r="E79" s="196">
+        <f>IF(FAR!H46="","",FAR!H46)</f>
+        <v/>
+      </c>
+      <c r="F79" s="197">
+        <f>IF(FAR!I46="","",FAR!I46)</f>
+        <v/>
+      </c>
+      <c r="G79" s="198">
+        <f>IF(FAR!K46="","",IFERROR(INDEX(FAR!$AA46:$BF46,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K46))</f>
+        <v/>
+      </c>
+      <c r="H79" s="199">
+        <f>IF(FAR!K46="",0,IF(AND(FAR!H46&lt;&gt;"",FAR!H46&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I46="",FAR!I46&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I79" s="175">
+        <f>IF($H79=1,FAR!K46,0)</f>
+        <v/>
+      </c>
+      <c r="J79" s="175">
+        <f>IF(AND(FAR!H46&lt;&gt;"",FAR!H46&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H46&lt;=ReportingFYEnd),FAR!K46,0)</f>
+        <v/>
+      </c>
+      <c r="K79" s="198">
+        <f>IF(AND(FAR!I46&lt;&gt;"",FAR!I46&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I46&lt;=ReportingFYEnd),FAR!K46,0)</f>
+        <v/>
+      </c>
+      <c r="L79" s="175">
+        <f>IF($H79=1,FAR!K46-$G79,0)</f>
+        <v/>
+      </c>
+      <c r="M79" s="175">
+        <f>IF(FAR!K46="",0,FAR!R46)</f>
+        <v/>
+      </c>
+      <c r="N79" s="199">
+        <f>IF(AND(FAR!I46&lt;&gt;"",FAR!I46&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I46&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O79" s="198">
+        <f>IF($N79=1,$L79+$M79,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="188">
+        <f>IF(FAR!K47="","",FAR!B47)</f>
+        <v/>
+      </c>
+      <c r="C80" s="189">
+        <f>IF(FAR!K47="","",FAR!C47)</f>
+        <v/>
+      </c>
+      <c r="D80" s="171">
+        <f>IF(FAR!K47="","",FAR!K47)</f>
+        <v/>
+      </c>
+      <c r="E80" s="190">
+        <f>IF(FAR!H47="","",FAR!H47)</f>
+        <v/>
+      </c>
+      <c r="F80" s="191">
+        <f>IF(FAR!I47="","",FAR!I47)</f>
+        <v/>
+      </c>
+      <c r="G80" s="192">
+        <f>IF(FAR!K47="","",IFERROR(INDEX(FAR!$AA47:$BF47,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K47))</f>
+        <v/>
+      </c>
+      <c r="H80" s="193">
+        <f>IF(FAR!K47="",0,IF(AND(FAR!H47&lt;&gt;"",FAR!H47&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I47="",FAR!I47&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I80" s="171">
+        <f>IF($H80=1,FAR!K47,0)</f>
+        <v/>
+      </c>
+      <c r="J80" s="171">
+        <f>IF(AND(FAR!H47&lt;&gt;"",FAR!H47&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H47&lt;=ReportingFYEnd),FAR!K47,0)</f>
+        <v/>
+      </c>
+      <c r="K80" s="192">
+        <f>IF(AND(FAR!I47&lt;&gt;"",FAR!I47&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I47&lt;=ReportingFYEnd),FAR!K47,0)</f>
+        <v/>
+      </c>
+      <c r="L80" s="171">
+        <f>IF($H80=1,FAR!K47-$G80,0)</f>
+        <v/>
+      </c>
+      <c r="M80" s="171">
+        <f>IF(FAR!K47="",0,FAR!R47)</f>
+        <v/>
+      </c>
+      <c r="N80" s="193">
+        <f>IF(AND(FAR!I47&lt;&gt;"",FAR!I47&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I47&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O80" s="192">
+        <f>IF($N80=1,$L80+$M80,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="194">
+        <f>IF(FAR!K48="","",FAR!B48)</f>
+        <v/>
+      </c>
+      <c r="C81" s="195">
+        <f>IF(FAR!K48="","",FAR!C48)</f>
+        <v/>
+      </c>
+      <c r="D81" s="175">
+        <f>IF(FAR!K48="","",FAR!K48)</f>
+        <v/>
+      </c>
+      <c r="E81" s="196">
+        <f>IF(FAR!H48="","",FAR!H48)</f>
+        <v/>
+      </c>
+      <c r="F81" s="197">
+        <f>IF(FAR!I48="","",FAR!I48)</f>
+        <v/>
+      </c>
+      <c r="G81" s="198">
+        <f>IF(FAR!K48="","",IFERROR(INDEX(FAR!$AA48:$BF48,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K48))</f>
+        <v/>
+      </c>
+      <c r="H81" s="199">
+        <f>IF(FAR!K48="",0,IF(AND(FAR!H48&lt;&gt;"",FAR!H48&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I48="",FAR!I48&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I81" s="175">
+        <f>IF($H81=1,FAR!K48,0)</f>
+        <v/>
+      </c>
+      <c r="J81" s="175">
+        <f>IF(AND(FAR!H48&lt;&gt;"",FAR!H48&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H48&lt;=ReportingFYEnd),FAR!K48,0)</f>
+        <v/>
+      </c>
+      <c r="K81" s="198">
+        <f>IF(AND(FAR!I48&lt;&gt;"",FAR!I48&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I48&lt;=ReportingFYEnd),FAR!K48,0)</f>
+        <v/>
+      </c>
+      <c r="L81" s="175">
+        <f>IF($H81=1,FAR!K48-$G81,0)</f>
+        <v/>
+      </c>
+      <c r="M81" s="175">
+        <f>IF(FAR!K48="",0,FAR!R48)</f>
+        <v/>
+      </c>
+      <c r="N81" s="199">
+        <f>IF(AND(FAR!I48&lt;&gt;"",FAR!I48&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I48&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O81" s="198">
+        <f>IF($N81=1,$L81+$M81,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="188">
+        <f>IF(FAR!K49="","",FAR!B49)</f>
+        <v/>
+      </c>
+      <c r="C82" s="189">
+        <f>IF(FAR!K49="","",FAR!C49)</f>
+        <v/>
+      </c>
+      <c r="D82" s="171">
+        <f>IF(FAR!K49="","",FAR!K49)</f>
+        <v/>
+      </c>
+      <c r="E82" s="190">
+        <f>IF(FAR!H49="","",FAR!H49)</f>
+        <v/>
+      </c>
+      <c r="F82" s="191">
+        <f>IF(FAR!I49="","",FAR!I49)</f>
+        <v/>
+      </c>
+      <c r="G82" s="192">
+        <f>IF(FAR!K49="","",IFERROR(INDEX(FAR!$AA49:$BF49,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K49))</f>
+        <v/>
+      </c>
+      <c r="H82" s="193">
+        <f>IF(FAR!K49="",0,IF(AND(FAR!H49&lt;&gt;"",FAR!H49&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I49="",FAR!I49&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I82" s="171">
+        <f>IF($H82=1,FAR!K49,0)</f>
+        <v/>
+      </c>
+      <c r="J82" s="171">
+        <f>IF(AND(FAR!H49&lt;&gt;"",FAR!H49&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H49&lt;=ReportingFYEnd),FAR!K49,0)</f>
+        <v/>
+      </c>
+      <c r="K82" s="192">
+        <f>IF(AND(FAR!I49&lt;&gt;"",FAR!I49&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I49&lt;=ReportingFYEnd),FAR!K49,0)</f>
+        <v/>
+      </c>
+      <c r="L82" s="171">
+        <f>IF($H82=1,FAR!K49-$G82,0)</f>
+        <v/>
+      </c>
+      <c r="M82" s="171">
+        <f>IF(FAR!K49="",0,FAR!R49)</f>
+        <v/>
+      </c>
+      <c r="N82" s="193">
+        <f>IF(AND(FAR!I49&lt;&gt;"",FAR!I49&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I49&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O82" s="192">
+        <f>IF($N82=1,$L82+$M82,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="194">
+        <f>IF(FAR!K50="","",FAR!B50)</f>
+        <v/>
+      </c>
+      <c r="C83" s="195">
+        <f>IF(FAR!K50="","",FAR!C50)</f>
+        <v/>
+      </c>
+      <c r="D83" s="175">
+        <f>IF(FAR!K50="","",FAR!K50)</f>
+        <v/>
+      </c>
+      <c r="E83" s="196">
+        <f>IF(FAR!H50="","",FAR!H50)</f>
+        <v/>
+      </c>
+      <c r="F83" s="197">
+        <f>IF(FAR!I50="","",FAR!I50)</f>
+        <v/>
+      </c>
+      <c r="G83" s="198">
+        <f>IF(FAR!K50="","",IFERROR(INDEX(FAR!$AA50:$BF50,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K50))</f>
+        <v/>
+      </c>
+      <c r="H83" s="199">
+        <f>IF(FAR!K50="",0,IF(AND(FAR!H50&lt;&gt;"",FAR!H50&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I50="",FAR!I50&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I83" s="175">
+        <f>IF($H83=1,FAR!K50,0)</f>
+        <v/>
+      </c>
+      <c r="J83" s="175">
+        <f>IF(AND(FAR!H50&lt;&gt;"",FAR!H50&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H50&lt;=ReportingFYEnd),FAR!K50,0)</f>
+        <v/>
+      </c>
+      <c r="K83" s="198">
+        <f>IF(AND(FAR!I50&lt;&gt;"",FAR!I50&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I50&lt;=ReportingFYEnd),FAR!K50,0)</f>
+        <v/>
+      </c>
+      <c r="L83" s="175">
+        <f>IF($H83=1,FAR!K50-$G83,0)</f>
+        <v/>
+      </c>
+      <c r="M83" s="175">
+        <f>IF(FAR!K50="",0,FAR!R50)</f>
+        <v/>
+      </c>
+      <c r="N83" s="199">
+        <f>IF(AND(FAR!I50&lt;&gt;"",FAR!I50&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I50&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O83" s="198">
+        <f>IF($N83=1,$L83+$M83,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="188">
+        <f>IF(FAR!K51="","",FAR!B51)</f>
+        <v/>
+      </c>
+      <c r="C84" s="189">
+        <f>IF(FAR!K51="","",FAR!C51)</f>
+        <v/>
+      </c>
+      <c r="D84" s="171">
+        <f>IF(FAR!K51="","",FAR!K51)</f>
+        <v/>
+      </c>
+      <c r="E84" s="190">
+        <f>IF(FAR!H51="","",FAR!H51)</f>
+        <v/>
+      </c>
+      <c r="F84" s="191">
+        <f>IF(FAR!I51="","",FAR!I51)</f>
+        <v/>
+      </c>
+      <c r="G84" s="192">
+        <f>IF(FAR!K51="","",IFERROR(INDEX(FAR!$AA51:$BF51,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K51))</f>
+        <v/>
+      </c>
+      <c r="H84" s="193">
+        <f>IF(FAR!K51="",0,IF(AND(FAR!H51&lt;&gt;"",FAR!H51&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I51="",FAR!I51&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I84" s="171">
+        <f>IF($H84=1,FAR!K51,0)</f>
+        <v/>
+      </c>
+      <c r="J84" s="171">
+        <f>IF(AND(FAR!H51&lt;&gt;"",FAR!H51&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H51&lt;=ReportingFYEnd),FAR!K51,0)</f>
+        <v/>
+      </c>
+      <c r="K84" s="192">
+        <f>IF(AND(FAR!I51&lt;&gt;"",FAR!I51&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I51&lt;=ReportingFYEnd),FAR!K51,0)</f>
+        <v/>
+      </c>
+      <c r="L84" s="171">
+        <f>IF($H84=1,FAR!K51-$G84,0)</f>
+        <v/>
+      </c>
+      <c r="M84" s="171">
+        <f>IF(FAR!K51="",0,FAR!R51)</f>
+        <v/>
+      </c>
+      <c r="N84" s="193">
+        <f>IF(AND(FAR!I51&lt;&gt;"",FAR!I51&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I51&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O84" s="192">
+        <f>IF($N84=1,$L84+$M84,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="194">
+        <f>IF(FAR!K52="","",FAR!B52)</f>
+        <v/>
+      </c>
+      <c r="C85" s="195">
+        <f>IF(FAR!K52="","",FAR!C52)</f>
+        <v/>
+      </c>
+      <c r="D85" s="175">
+        <f>IF(FAR!K52="","",FAR!K52)</f>
+        <v/>
+      </c>
+      <c r="E85" s="196">
+        <f>IF(FAR!H52="","",FAR!H52)</f>
+        <v/>
+      </c>
+      <c r="F85" s="197">
+        <f>IF(FAR!I52="","",FAR!I52)</f>
+        <v/>
+      </c>
+      <c r="G85" s="198">
+        <f>IF(FAR!K52="","",IFERROR(INDEX(FAR!$AA52:$BF52,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K52))</f>
+        <v/>
+      </c>
+      <c r="H85" s="199">
+        <f>IF(FAR!K52="",0,IF(AND(FAR!H52&lt;&gt;"",FAR!H52&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I52="",FAR!I52&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I85" s="175">
+        <f>IF($H85=1,FAR!K52,0)</f>
+        <v/>
+      </c>
+      <c r="J85" s="175">
+        <f>IF(AND(FAR!H52&lt;&gt;"",FAR!H52&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H52&lt;=ReportingFYEnd),FAR!K52,0)</f>
+        <v/>
+      </c>
+      <c r="K85" s="198">
+        <f>IF(AND(FAR!I52&lt;&gt;"",FAR!I52&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I52&lt;=ReportingFYEnd),FAR!K52,0)</f>
+        <v/>
+      </c>
+      <c r="L85" s="175">
+        <f>IF($H85=1,FAR!K52-$G85,0)</f>
+        <v/>
+      </c>
+      <c r="M85" s="175">
+        <f>IF(FAR!K52="",0,FAR!R52)</f>
+        <v/>
+      </c>
+      <c r="N85" s="199">
+        <f>IF(AND(FAR!I52&lt;&gt;"",FAR!I52&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I52&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O85" s="198">
+        <f>IF($N85=1,$L85+$M85,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="188">
+        <f>IF(FAR!K53="","",FAR!B53)</f>
+        <v/>
+      </c>
+      <c r="C86" s="189">
+        <f>IF(FAR!K53="","",FAR!C53)</f>
+        <v/>
+      </c>
+      <c r="D86" s="171">
+        <f>IF(FAR!K53="","",FAR!K53)</f>
+        <v/>
+      </c>
+      <c r="E86" s="190">
+        <f>IF(FAR!H53="","",FAR!H53)</f>
+        <v/>
+      </c>
+      <c r="F86" s="191">
+        <f>IF(FAR!I53="","",FAR!I53)</f>
+        <v/>
+      </c>
+      <c r="G86" s="192">
+        <f>IF(FAR!K53="","",IFERROR(INDEX(FAR!$AA53:$BF53,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K53))</f>
+        <v/>
+      </c>
+      <c r="H86" s="193">
+        <f>IF(FAR!K53="",0,IF(AND(FAR!H53&lt;&gt;"",FAR!H53&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I53="",FAR!I53&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I86" s="171">
+        <f>IF($H86=1,FAR!K53,0)</f>
+        <v/>
+      </c>
+      <c r="J86" s="171">
+        <f>IF(AND(FAR!H53&lt;&gt;"",FAR!H53&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H53&lt;=ReportingFYEnd),FAR!K53,0)</f>
+        <v/>
+      </c>
+      <c r="K86" s="192">
+        <f>IF(AND(FAR!I53&lt;&gt;"",FAR!I53&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I53&lt;=ReportingFYEnd),FAR!K53,0)</f>
+        <v/>
+      </c>
+      <c r="L86" s="171">
+        <f>IF($H86=1,FAR!K53-$G86,0)</f>
+        <v/>
+      </c>
+      <c r="M86" s="171">
+        <f>IF(FAR!K53="",0,FAR!R53)</f>
+        <v/>
+      </c>
+      <c r="N86" s="193">
+        <f>IF(AND(FAR!I53&lt;&gt;"",FAR!I53&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I53&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O86" s="192">
+        <f>IF($N86=1,$L86+$M86,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="194">
+        <f>IF(FAR!K54="","",FAR!B54)</f>
+        <v/>
+      </c>
+      <c r="C87" s="195">
+        <f>IF(FAR!K54="","",FAR!C54)</f>
+        <v/>
+      </c>
+      <c r="D87" s="175">
+        <f>IF(FAR!K54="","",FAR!K54)</f>
+        <v/>
+      </c>
+      <c r="E87" s="196">
+        <f>IF(FAR!H54="","",FAR!H54)</f>
+        <v/>
+      </c>
+      <c r="F87" s="197">
+        <f>IF(FAR!I54="","",FAR!I54)</f>
+        <v/>
+      </c>
+      <c r="G87" s="198">
+        <f>IF(FAR!K54="","",IFERROR(INDEX(FAR!$AA54:$BF54,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K54))</f>
+        <v/>
+      </c>
+      <c r="H87" s="199">
+        <f>IF(FAR!K54="",0,IF(AND(FAR!H54&lt;&gt;"",FAR!H54&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I54="",FAR!I54&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I87" s="175">
+        <f>IF($H87=1,FAR!K54,0)</f>
+        <v/>
+      </c>
+      <c r="J87" s="175">
+        <f>IF(AND(FAR!H54&lt;&gt;"",FAR!H54&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H54&lt;=ReportingFYEnd),FAR!K54,0)</f>
+        <v/>
+      </c>
+      <c r="K87" s="198">
+        <f>IF(AND(FAR!I54&lt;&gt;"",FAR!I54&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I54&lt;=ReportingFYEnd),FAR!K54,0)</f>
+        <v/>
+      </c>
+      <c r="L87" s="175">
+        <f>IF($H87=1,FAR!K54-$G87,0)</f>
+        <v/>
+      </c>
+      <c r="M87" s="175">
+        <f>IF(FAR!K54="",0,FAR!R54)</f>
+        <v/>
+      </c>
+      <c r="N87" s="199">
+        <f>IF(AND(FAR!I54&lt;&gt;"",FAR!I54&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I54&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O87" s="198">
+        <f>IF($N87=1,$L87+$M87,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="188">
+        <f>IF(FAR!K55="","",FAR!B55)</f>
+        <v/>
+      </c>
+      <c r="C88" s="189">
+        <f>IF(FAR!K55="","",FAR!C55)</f>
+        <v/>
+      </c>
+      <c r="D88" s="171">
+        <f>IF(FAR!K55="","",FAR!K55)</f>
+        <v/>
+      </c>
+      <c r="E88" s="190">
+        <f>IF(FAR!H55="","",FAR!H55)</f>
+        <v/>
+      </c>
+      <c r="F88" s="191">
+        <f>IF(FAR!I55="","",FAR!I55)</f>
+        <v/>
+      </c>
+      <c r="G88" s="192">
+        <f>IF(FAR!K55="","",IFERROR(INDEX(FAR!$AA55:$BF55,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K55))</f>
+        <v/>
+      </c>
+      <c r="H88" s="193">
+        <f>IF(FAR!K55="",0,IF(AND(FAR!H55&lt;&gt;"",FAR!H55&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I55="",FAR!I55&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I88" s="171">
+        <f>IF($H88=1,FAR!K55,0)</f>
+        <v/>
+      </c>
+      <c r="J88" s="171">
+        <f>IF(AND(FAR!H55&lt;&gt;"",FAR!H55&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H55&lt;=ReportingFYEnd),FAR!K55,0)</f>
+        <v/>
+      </c>
+      <c r="K88" s="192">
+        <f>IF(AND(FAR!I55&lt;&gt;"",FAR!I55&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I55&lt;=ReportingFYEnd),FAR!K55,0)</f>
+        <v/>
+      </c>
+      <c r="L88" s="171">
+        <f>IF($H88=1,FAR!K55-$G88,0)</f>
+        <v/>
+      </c>
+      <c r="M88" s="171">
+        <f>IF(FAR!K55="",0,FAR!R55)</f>
+        <v/>
+      </c>
+      <c r="N88" s="193">
+        <f>IF(AND(FAR!I55&lt;&gt;"",FAR!I55&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I55&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O88" s="192">
+        <f>IF($N88=1,$L88+$M88,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="194">
+        <f>IF(FAR!K56="","",FAR!B56)</f>
+        <v/>
+      </c>
+      <c r="C89" s="195">
+        <f>IF(FAR!K56="","",FAR!C56)</f>
+        <v/>
+      </c>
+      <c r="D89" s="175">
+        <f>IF(FAR!K56="","",FAR!K56)</f>
+        <v/>
+      </c>
+      <c r="E89" s="196">
+        <f>IF(FAR!H56="","",FAR!H56)</f>
+        <v/>
+      </c>
+      <c r="F89" s="197">
+        <f>IF(FAR!I56="","",FAR!I56)</f>
+        <v/>
+      </c>
+      <c r="G89" s="198">
+        <f>IF(FAR!K56="","",IFERROR(INDEX(FAR!$AA56:$BF56,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K56))</f>
+        <v/>
+      </c>
+      <c r="H89" s="199">
+        <f>IF(FAR!K56="",0,IF(AND(FAR!H56&lt;&gt;"",FAR!H56&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I56="",FAR!I56&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I89" s="175">
+        <f>IF($H89=1,FAR!K56,0)</f>
+        <v/>
+      </c>
+      <c r="J89" s="175">
+        <f>IF(AND(FAR!H56&lt;&gt;"",FAR!H56&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H56&lt;=ReportingFYEnd),FAR!K56,0)</f>
+        <v/>
+      </c>
+      <c r="K89" s="198">
+        <f>IF(AND(FAR!I56&lt;&gt;"",FAR!I56&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I56&lt;=ReportingFYEnd),FAR!K56,0)</f>
+        <v/>
+      </c>
+      <c r="L89" s="175">
+        <f>IF($H89=1,FAR!K56-$G89,0)</f>
+        <v/>
+      </c>
+      <c r="M89" s="175">
+        <f>IF(FAR!K56="",0,FAR!R56)</f>
+        <v/>
+      </c>
+      <c r="N89" s="199">
+        <f>IF(AND(FAR!I56&lt;&gt;"",FAR!I56&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I56&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O89" s="198">
+        <f>IF($N89=1,$L89+$M89,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="188">
+        <f>IF(FAR!K57="","",FAR!B57)</f>
+        <v/>
+      </c>
+      <c r="C90" s="189">
+        <f>IF(FAR!K57="","",FAR!C57)</f>
+        <v/>
+      </c>
+      <c r="D90" s="171">
+        <f>IF(FAR!K57="","",FAR!K57)</f>
+        <v/>
+      </c>
+      <c r="E90" s="190">
+        <f>IF(FAR!H57="","",FAR!H57)</f>
+        <v/>
+      </c>
+      <c r="F90" s="191">
+        <f>IF(FAR!I57="","",FAR!I57)</f>
+        <v/>
+      </c>
+      <c r="G90" s="192">
+        <f>IF(FAR!K57="","",IFERROR(INDEX(FAR!$AA57:$BF57,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K57))</f>
+        <v/>
+      </c>
+      <c r="H90" s="193">
+        <f>IF(FAR!K57="",0,IF(AND(FAR!H57&lt;&gt;"",FAR!H57&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I57="",FAR!I57&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I90" s="171">
+        <f>IF($H90=1,FAR!K57,0)</f>
+        <v/>
+      </c>
+      <c r="J90" s="171">
+        <f>IF(AND(FAR!H57&lt;&gt;"",FAR!H57&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H57&lt;=ReportingFYEnd),FAR!K57,0)</f>
+        <v/>
+      </c>
+      <c r="K90" s="192">
+        <f>IF(AND(FAR!I57&lt;&gt;"",FAR!I57&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I57&lt;=ReportingFYEnd),FAR!K57,0)</f>
+        <v/>
+      </c>
+      <c r="L90" s="171">
+        <f>IF($H90=1,FAR!K57-$G90,0)</f>
+        <v/>
+      </c>
+      <c r="M90" s="171">
+        <f>IF(FAR!K57="",0,FAR!R57)</f>
+        <v/>
+      </c>
+      <c r="N90" s="193">
+        <f>IF(AND(FAR!I57&lt;&gt;"",FAR!I57&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I57&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O90" s="192">
+        <f>IF($N90=1,$L90+$M90,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="194">
+        <f>IF(FAR!K58="","",FAR!B58)</f>
+        <v/>
+      </c>
+      <c r="C91" s="195">
+        <f>IF(FAR!K58="","",FAR!C58)</f>
+        <v/>
+      </c>
+      <c r="D91" s="175">
+        <f>IF(FAR!K58="","",FAR!K58)</f>
+        <v/>
+      </c>
+      <c r="E91" s="196">
+        <f>IF(FAR!H58="","",FAR!H58)</f>
+        <v/>
+      </c>
+      <c r="F91" s="197">
+        <f>IF(FAR!I58="","",FAR!I58)</f>
+        <v/>
+      </c>
+      <c r="G91" s="198">
+        <f>IF(FAR!K58="","",IFERROR(INDEX(FAR!$AA58:$BF58,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K58))</f>
+        <v/>
+      </c>
+      <c r="H91" s="199">
+        <f>IF(FAR!K58="",0,IF(AND(FAR!H58&lt;&gt;"",FAR!H58&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I58="",FAR!I58&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I91" s="175">
+        <f>IF($H91=1,FAR!K58,0)</f>
+        <v/>
+      </c>
+      <c r="J91" s="175">
+        <f>IF(AND(FAR!H58&lt;&gt;"",FAR!H58&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H58&lt;=ReportingFYEnd),FAR!K58,0)</f>
+        <v/>
+      </c>
+      <c r="K91" s="198">
+        <f>IF(AND(FAR!I58&lt;&gt;"",FAR!I58&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I58&lt;=ReportingFYEnd),FAR!K58,0)</f>
+        <v/>
+      </c>
+      <c r="L91" s="175">
+        <f>IF($H91=1,FAR!K58-$G91,0)</f>
+        <v/>
+      </c>
+      <c r="M91" s="175">
+        <f>IF(FAR!K58="",0,FAR!R58)</f>
+        <v/>
+      </c>
+      <c r="N91" s="199">
+        <f>IF(AND(FAR!I58&lt;&gt;"",FAR!I58&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I58&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O91" s="198">
+        <f>IF($N91=1,$L91+$M91,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="188">
+        <f>IF(FAR!K59="","",FAR!B59)</f>
+        <v/>
+      </c>
+      <c r="C92" s="189">
+        <f>IF(FAR!K59="","",FAR!C59)</f>
+        <v/>
+      </c>
+      <c r="D92" s="171">
+        <f>IF(FAR!K59="","",FAR!K59)</f>
+        <v/>
+      </c>
+      <c r="E92" s="190">
+        <f>IF(FAR!H59="","",FAR!H59)</f>
+        <v/>
+      </c>
+      <c r="F92" s="191">
+        <f>IF(FAR!I59="","",FAR!I59)</f>
+        <v/>
+      </c>
+      <c r="G92" s="192">
+        <f>IF(FAR!K59="","",IFERROR(INDEX(FAR!$AA59:$BF59,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K59))</f>
+        <v/>
+      </c>
+      <c r="H92" s="193">
+        <f>IF(FAR!K59="",0,IF(AND(FAR!H59&lt;&gt;"",FAR!H59&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I59="",FAR!I59&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I92" s="171">
+        <f>IF($H92=1,FAR!K59,0)</f>
+        <v/>
+      </c>
+      <c r="J92" s="171">
+        <f>IF(AND(FAR!H59&lt;&gt;"",FAR!H59&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H59&lt;=ReportingFYEnd),FAR!K59,0)</f>
+        <v/>
+      </c>
+      <c r="K92" s="192">
+        <f>IF(AND(FAR!I59&lt;&gt;"",FAR!I59&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I59&lt;=ReportingFYEnd),FAR!K59,0)</f>
+        <v/>
+      </c>
+      <c r="L92" s="171">
+        <f>IF($H92=1,FAR!K59-$G92,0)</f>
+        <v/>
+      </c>
+      <c r="M92" s="171">
+        <f>IF(FAR!K59="",0,FAR!R59)</f>
+        <v/>
+      </c>
+      <c r="N92" s="193">
+        <f>IF(AND(FAR!I59&lt;&gt;"",FAR!I59&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I59&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O92" s="192">
+        <f>IF($N92=1,$L92+$M92,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="194">
+        <f>IF(FAR!K60="","",FAR!B60)</f>
+        <v/>
+      </c>
+      <c r="C93" s="195">
+        <f>IF(FAR!K60="","",FAR!C60)</f>
+        <v/>
+      </c>
+      <c r="D93" s="175">
+        <f>IF(FAR!K60="","",FAR!K60)</f>
+        <v/>
+      </c>
+      <c r="E93" s="196">
+        <f>IF(FAR!H60="","",FAR!H60)</f>
+        <v/>
+      </c>
+      <c r="F93" s="197">
+        <f>IF(FAR!I60="","",FAR!I60)</f>
+        <v/>
+      </c>
+      <c r="G93" s="198">
+        <f>IF(FAR!K60="","",IFERROR(INDEX(FAR!$AA60:$BF60,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K60))</f>
+        <v/>
+      </c>
+      <c r="H93" s="199">
+        <f>IF(FAR!K60="",0,IF(AND(FAR!H60&lt;&gt;"",FAR!H60&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I60="",FAR!I60&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I93" s="175">
+        <f>IF($H93=1,FAR!K60,0)</f>
+        <v/>
+      </c>
+      <c r="J93" s="175">
+        <f>IF(AND(FAR!H60&lt;&gt;"",FAR!H60&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H60&lt;=ReportingFYEnd),FAR!K60,0)</f>
+        <v/>
+      </c>
+      <c r="K93" s="198">
+        <f>IF(AND(FAR!I60&lt;&gt;"",FAR!I60&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I60&lt;=ReportingFYEnd),FAR!K60,0)</f>
+        <v/>
+      </c>
+      <c r="L93" s="175">
+        <f>IF($H93=1,FAR!K60-$G93,0)</f>
+        <v/>
+      </c>
+      <c r="M93" s="175">
+        <f>IF(FAR!K60="",0,FAR!R60)</f>
+        <v/>
+      </c>
+      <c r="N93" s="199">
+        <f>IF(AND(FAR!I60&lt;&gt;"",FAR!I60&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I60&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O93" s="198">
+        <f>IF($N93=1,$L93+$M93,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="188">
+        <f>IF(FAR!K61="","",FAR!B61)</f>
+        <v/>
+      </c>
+      <c r="C94" s="189">
+        <f>IF(FAR!K61="","",FAR!C61)</f>
+        <v/>
+      </c>
+      <c r="D94" s="171">
+        <f>IF(FAR!K61="","",FAR!K61)</f>
+        <v/>
+      </c>
+      <c r="E94" s="190">
+        <f>IF(FAR!H61="","",FAR!H61)</f>
+        <v/>
+      </c>
+      <c r="F94" s="191">
+        <f>IF(FAR!I61="","",FAR!I61)</f>
+        <v/>
+      </c>
+      <c r="G94" s="192">
+        <f>IF(FAR!K61="","",IFERROR(INDEX(FAR!$AA61:$BF61,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K61))</f>
+        <v/>
+      </c>
+      <c r="H94" s="193">
+        <f>IF(FAR!K61="",0,IF(AND(FAR!H61&lt;&gt;"",FAR!H61&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I61="",FAR!I61&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I94" s="171">
+        <f>IF($H94=1,FAR!K61,0)</f>
+        <v/>
+      </c>
+      <c r="J94" s="171">
+        <f>IF(AND(FAR!H61&lt;&gt;"",FAR!H61&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H61&lt;=ReportingFYEnd),FAR!K61,0)</f>
+        <v/>
+      </c>
+      <c r="K94" s="192">
+        <f>IF(AND(FAR!I61&lt;&gt;"",FAR!I61&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I61&lt;=ReportingFYEnd),FAR!K61,0)</f>
+        <v/>
+      </c>
+      <c r="L94" s="171">
+        <f>IF($H94=1,FAR!K61-$G94,0)</f>
+        <v/>
+      </c>
+      <c r="M94" s="171">
+        <f>IF(FAR!K61="",0,FAR!R61)</f>
+        <v/>
+      </c>
+      <c r="N94" s="193">
+        <f>IF(AND(FAR!I61&lt;&gt;"",FAR!I61&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I61&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O94" s="192">
+        <f>IF($N94=1,$L94+$M94,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="194">
+        <f>IF(FAR!K62="","",FAR!B62)</f>
+        <v/>
+      </c>
+      <c r="C95" s="195">
+        <f>IF(FAR!K62="","",FAR!C62)</f>
+        <v/>
+      </c>
+      <c r="D95" s="175">
+        <f>IF(FAR!K62="","",FAR!K62)</f>
+        <v/>
+      </c>
+      <c r="E95" s="196">
+        <f>IF(FAR!H62="","",FAR!H62)</f>
+        <v/>
+      </c>
+      <c r="F95" s="197">
+        <f>IF(FAR!I62="","",FAR!I62)</f>
+        <v/>
+      </c>
+      <c r="G95" s="198">
+        <f>IF(FAR!K62="","",IFERROR(INDEX(FAR!$AA62:$BF62,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K62))</f>
+        <v/>
+      </c>
+      <c r="H95" s="199">
+        <f>IF(FAR!K62="",0,IF(AND(FAR!H62&lt;&gt;"",FAR!H62&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I62="",FAR!I62&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I95" s="175">
+        <f>IF($H95=1,FAR!K62,0)</f>
+        <v/>
+      </c>
+      <c r="J95" s="175">
+        <f>IF(AND(FAR!H62&lt;&gt;"",FAR!H62&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H62&lt;=ReportingFYEnd),FAR!K62,0)</f>
+        <v/>
+      </c>
+      <c r="K95" s="198">
+        <f>IF(AND(FAR!I62&lt;&gt;"",FAR!I62&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I62&lt;=ReportingFYEnd),FAR!K62,0)</f>
+        <v/>
+      </c>
+      <c r="L95" s="175">
+        <f>IF($H95=1,FAR!K62-$G95,0)</f>
+        <v/>
+      </c>
+      <c r="M95" s="175">
+        <f>IF(FAR!K62="",0,FAR!R62)</f>
+        <v/>
+      </c>
+      <c r="N95" s="199">
+        <f>IF(AND(FAR!I62&lt;&gt;"",FAR!I62&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I62&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O95" s="198">
+        <f>IF($N95=1,$L95+$M95,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="188">
+        <f>IF(FAR!K63="","",FAR!B63)</f>
+        <v/>
+      </c>
+      <c r="C96" s="189">
+        <f>IF(FAR!K63="","",FAR!C63)</f>
+        <v/>
+      </c>
+      <c r="D96" s="171">
+        <f>IF(FAR!K63="","",FAR!K63)</f>
+        <v/>
+      </c>
+      <c r="E96" s="190">
+        <f>IF(FAR!H63="","",FAR!H63)</f>
+        <v/>
+      </c>
+      <c r="F96" s="191">
+        <f>IF(FAR!I63="","",FAR!I63)</f>
+        <v/>
+      </c>
+      <c r="G96" s="192">
+        <f>IF(FAR!K63="","",IFERROR(INDEX(FAR!$AA63:$BF63,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K63))</f>
+        <v/>
+      </c>
+      <c r="H96" s="193">
+        <f>IF(FAR!K63="",0,IF(AND(FAR!H63&lt;&gt;"",FAR!H63&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I63="",FAR!I63&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I96" s="171">
+        <f>IF($H96=1,FAR!K63,0)</f>
+        <v/>
+      </c>
+      <c r="J96" s="171">
+        <f>IF(AND(FAR!H63&lt;&gt;"",FAR!H63&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H63&lt;=ReportingFYEnd),FAR!K63,0)</f>
+        <v/>
+      </c>
+      <c r="K96" s="192">
+        <f>IF(AND(FAR!I63&lt;&gt;"",FAR!I63&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I63&lt;=ReportingFYEnd),FAR!K63,0)</f>
+        <v/>
+      </c>
+      <c r="L96" s="171">
+        <f>IF($H96=1,FAR!K63-$G96,0)</f>
+        <v/>
+      </c>
+      <c r="M96" s="171">
+        <f>IF(FAR!K63="",0,FAR!R63)</f>
+        <v/>
+      </c>
+      <c r="N96" s="193">
+        <f>IF(AND(FAR!I63&lt;&gt;"",FAR!I63&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I63&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O96" s="192">
+        <f>IF($N96=1,$L96+$M96,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="194">
+        <f>IF(FAR!K64="","",FAR!B64)</f>
+        <v/>
+      </c>
+      <c r="C97" s="195">
+        <f>IF(FAR!K64="","",FAR!C64)</f>
+        <v/>
+      </c>
+      <c r="D97" s="175">
+        <f>IF(FAR!K64="","",FAR!K64)</f>
+        <v/>
+      </c>
+      <c r="E97" s="196">
+        <f>IF(FAR!H64="","",FAR!H64)</f>
+        <v/>
+      </c>
+      <c r="F97" s="197">
+        <f>IF(FAR!I64="","",FAR!I64)</f>
+        <v/>
+      </c>
+      <c r="G97" s="198">
+        <f>IF(FAR!K64="","",IFERROR(INDEX(FAR!$AA64:$BF64,MATCH(EDATE(ReportingFYEnd,-12),FAR!$AA$3:$BF$3,0)+1),FAR!K64))</f>
+        <v/>
+      </c>
+      <c r="H97" s="199">
+        <f>IF(FAR!K64="",0,IF(AND(FAR!H64&lt;&gt;"",FAR!H64&lt;=EDATE(ReportingFYEnd,-12),OR(FAR!I64="",FAR!I64&gt;EDATE(ReportingFYEnd,-12))),1,0))</f>
+        <v/>
+      </c>
+      <c r="I97" s="175">
+        <f>IF($H97=1,FAR!K64,0)</f>
+        <v/>
+      </c>
+      <c r="J97" s="175">
+        <f>IF(AND(FAR!H64&lt;&gt;"",FAR!H64&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!H64&lt;=ReportingFYEnd),FAR!K64,0)</f>
+        <v/>
+      </c>
+      <c r="K97" s="198">
+        <f>IF(AND(FAR!I64&lt;&gt;"",FAR!I64&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I64&lt;=ReportingFYEnd),FAR!K64,0)</f>
+        <v/>
+      </c>
+      <c r="L97" s="175">
+        <f>IF($H97=1,FAR!K64-$G97,0)</f>
+        <v/>
+      </c>
+      <c r="M97" s="175">
+        <f>IF(FAR!K64="",0,FAR!R64)</f>
+        <v/>
+      </c>
+      <c r="N97" s="199">
+        <f>IF(AND(FAR!I64&lt;&gt;"",FAR!I64&gt;=(EDATE(ReportingFYEnd,-12)+1),FAR!I64&lt;=ReportingFYEnd),1,0)</f>
+        <v/>
+      </c>
+      <c r="O97" s="198">
+        <f>IF($N97=1,$L97+$M97,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B29:L29"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="B36:O36"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="G5:J5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>